<commit_message>
Add Free & Paid Resources columns to M7 Year-1 curriculum master sheet
Added two new columns (K: Free Resources, L: Paid Resources) to all 41
course rows in the Master – By Topic sheet, mapping each HBS/MIT/Stanford
first-year course to the best available YouTube channels, MOOCs, and paid
HBS Online / Coursera equivalents.

https://claude.ai/code/session_011QHxcNSM1P2957ocCew2SU
</commit_message>
<xml_diff>
--- a/m7_year1_master_by_topic.xlsx
+++ b/m7_year1_master_by_topic.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master – By Topic" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Matrix" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Master – By Topic" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Coverage Matrix" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +59,13 @@
     <font>
       <color rgb="00BBBBBB"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -137,6 +142,11 @@
         <fgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -197,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -375,6 +385,90 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -754,6 +848,8 @@
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="52" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -821,1942 +917,2451 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="K3" s="62" t="inlineStr">
+        <is>
+          <t>Free Resources (YouTube / MOOCs)</t>
+        </is>
+      </c>
+      <c r="L3" s="62" t="inlineStr">
+        <is>
+          <t>Paid Resources (HBS Online / Coursera)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="63" t="inlineStr">
         <is>
           <t>Accounting</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="64" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="64" t="inlineStr">
         <is>
           <t>Financial Reporting and Control (FRC)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="64" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="64" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="64" t="inlineStr">
         <is>
           <t>Accounting &amp; Management</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="64" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="64" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="64" t="inlineStr">
         <is>
           <t>Accounting fundamentals: how to read, interpret, and use financial statements; managerial control systems.</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr"/>
+      <c r="J4" s="64" t="inlineStr"/>
+      <c r="K4" s="65" t="inlineStr">
+        <is>
+          <t>Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+MIT OCW Financial Accounting 15.515 (ocw.mit.edu/courses/15-515-financial-accounting-fall-2003/)
+Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)
+Farhat Accounting Lectures (YT: search 'Farhat Lectures')</t>
+        </is>
+      </c>
+      <c r="L4" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+HBS Online CORe Bundle ~$2,650 – includes Financial Accounting (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="66" t="n"/>
+      <c r="B5" s="64" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="64" t="inlineStr">
         <is>
           <t>Financial Accounting</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="64" t="inlineStr">
         <is>
           <t>15.501 / 15.516</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="64" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="64" t="inlineStr">
         <is>
           <t>Accounting</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="64" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="64" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="64" t="inlineStr">
         <is>
           <t>Reading/interpreting financial statements; accrual accounting, revenue recognition, balance-sheet analysis.</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr"/>
+      <c r="J5" s="64" t="inlineStr"/>
+      <c r="K5" s="65" t="inlineStr">
+        <is>
+          <t>Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+MIT OCW Financial Accounting 15.515 (ocw.mit.edu/courses/15-515-financial-accounting-fall-2003/)
+Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)</t>
+        </is>
+      </c>
+      <c r="L5" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="66" t="n"/>
+      <c r="B6" s="64" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="64" t="inlineStr">
         <is>
           <t>Financial Accounting</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="64" t="inlineStr">
         <is>
           <t>ACCT 210</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="64" t="inlineStr">
         <is>
           <t>Autumn</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="64" t="inlineStr">
         <is>
           <t>Analytical Foundations</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="64" t="inlineStr">
         <is>
           <t>4 units</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="64" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="64" t="inlineStr">
         <is>
           <t>How economic activities map into financial statements; balance sheets, income statements, cash flow.</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr"/>
+      <c r="J6" s="64" t="inlineStr"/>
+      <c r="K6" s="65" t="inlineStr">
+        <is>
+          <t>Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+MIT OCW Financial Accounting 15.515 (ocw.mit.edu/courses/15-515-financial-accounting-fall-2003/)
+Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)</t>
+        </is>
+      </c>
+      <c r="L6" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="67" t="n"/>
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>Managerial Accounting</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>ACCT 219</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="64" t="inlineStr">
         <is>
           <t>Spring</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="64" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="64" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="64" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="64" t="inlineStr">
         <is>
           <t>Using accounting information for internal decisions: cost accounting, budgeting, performance measurement.</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr"/>
+      <c r="J7" s="64" t="inlineStr"/>
+      <c r="K7" s="65" t="inlineStr">
+        <is>
+          <t>Edspira – Managerial Accounting series (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+Farhat Accounting Lectures – Managerial Accounting (YT: search 'Farhat Lectures')
+Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)</t>
+        </is>
+      </c>
+      <c r="L7" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="69" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="69" t="inlineStr">
         <is>
           <t>Finance I</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="69" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="69" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="69" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="69" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="69" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="I8" s="69" t="inlineStr">
         <is>
           <t>Foundations of financial analysis: valuation, capital markets, cost of capital, investment decisions.</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr"/>
+      <c r="J8" s="69" t="inlineStr"/>
+      <c r="K8" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Corporate Finance Full Course (YT: youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw)
+Patrick Boyle – On Finance (YT: youtube.com/@PBoyle)
+Corporate Finance Institute – CFI (YT: youtube.com/channel/UCGtbVv_ACgV7difdVZ92NMw)
+Khan Academy – Finance (khanacademy.org/economics-finance-domain/core-finance)</t>
+        </is>
+      </c>
+      <c r="L8" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
+HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="A9" s="66" t="n"/>
+      <c r="B9" s="69" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="69" t="inlineStr">
         <is>
           <t>Finance II</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="69" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="69" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="69" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="69" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="69" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="69" t="inlineStr">
         <is>
           <t>Advanced topics: capital structure, M&amp;A, corporate governance, financial policy.</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr"/>
+      <c r="J9" s="69" t="inlineStr"/>
+      <c r="K9" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Valuation Full Course (YT: youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw)
+Patrick Boyle – On Finance (YT: youtube.com/@PBoyle)
+Corporate Finance Institute – CFI (YT: youtube.com/channel/UCGtbVv_ACgV7difdVZ92NMw)</t>
+        </is>
+      </c>
+      <c r="L9" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="A10" s="66" t="n"/>
+      <c r="B10" s="69" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="69" t="inlineStr">
         <is>
           <t>Managerial Finance</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="69" t="inlineStr">
         <is>
           <t>15.401</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="69" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="69" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="69" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="69" t="inlineStr">
         <is>
           <t>Core Elective (choose 1 of 4)</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
+      <c r="I10" s="69" t="inlineStr">
         <is>
           <t>Corporate finance fundamentals: capital budgeting, valuation, risk, capital structure, financial markets.</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="69" t="inlineStr">
         <is>
           <t>One of 4 Sem-1 'core electives'</t>
         </is>
       </c>
+      <c r="K10" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Corporate Finance Full Course (YT: youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw)
+Patrick Boyle – On Finance (YT: youtube.com/@PBoyle)
+Corporate Finance Institute – CFI (YT: youtube.com/channel/UCGtbVv_ACgV7difdVZ92NMw)</t>
+        </is>
+      </c>
+      <c r="L10" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
+Wharton Finance on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="A11" s="67" t="n"/>
+      <c r="B11" s="69" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="69" t="inlineStr">
         <is>
           <t>Corporate Finance</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="69" t="inlineStr">
         <is>
           <t>FINANCE 229</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="69" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="69" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="69" t="inlineStr">
         <is>
           <t>4 units</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="H11" s="69" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
+      <c r="I11" s="69" t="inlineStr">
         <is>
           <t>Capital budgeting, valuation, risk and return, capital structure, corporate financial policy.</t>
         </is>
       </c>
-      <c r="J11" s="10" t="inlineStr"/>
+      <c r="J11" s="69" t="inlineStr"/>
+      <c r="K11" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Valuation MBA Spring 2025 (YT: youtube.com/playlist?list=PLUkh9m2BorqkgpNyRpP-NL3BS4yvFabXk)
+Patrick Boyle – On Finance (YT: youtube.com/@PBoyle)
+Corporate Finance Institute – CFI (YT: youtube.com/channel/UCGtbVv_ACgV7difdVZ92NMw)</t>
+        </is>
+      </c>
+      <c r="L11" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
+Wharton Finance on Coursera – free audit / $49 cert (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="70" t="inlineStr">
         <is>
           <t>Economics, Government &amp; Global Economy</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="71" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="71" t="inlineStr">
         <is>
           <t>Business, Government, and the International Economy (BGIE)</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="71" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="71" t="inlineStr">
         <is>
           <t>Economics &amp; Policy</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="G12" s="71" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="H12" s="71" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I12" s="13" t="inlineStr">
+      <c r="I12" s="71" t="inlineStr">
         <is>
           <t>Macroeconomics, trade policy, currency markets, political economy of business in a global context.</t>
         </is>
       </c>
-      <c r="J12" s="13" t="inlineStr">
+      <c r="J12" s="71" t="inlineStr">
         <is>
           <t>Macro / political economy</t>
         </is>
       </c>
+      <c r="K12" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Micro + Macro (mru.org / YT: youtube.com/channel/UCnkEhPBMZcEO0QGu51fDFDg)
+Freakonomics Radio Podcast – applied economics (freakonomics.com)
+Economics Explained (YT: youtube.com/c/EconomicsExplained)
+Khan Academy Macroeconomics (khanacademy.org/economics-finance-domain/macroeconomics)</t>
+        </is>
+      </c>
+      <c r="L12" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="A13" s="66" t="n"/>
+      <c r="B13" s="71" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="71" t="inlineStr">
         <is>
           <t>Economic Analysis for Business Decisions</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="71" t="inlineStr">
         <is>
           <t>15.010 / 15.011</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="71" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="71" t="inlineStr">
         <is>
           <t>Microeconomics</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="71" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="71" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="71" t="inlineStr">
         <is>
           <t>Applied micro: market structure, pricing, supply &amp; demand, game theory, strategic interaction.</t>
         </is>
       </c>
-      <c r="J13" s="13" t="inlineStr">
+      <c r="J13" s="71" t="inlineStr">
         <is>
           <t>Micro</t>
         </is>
       </c>
+      <c r="K13" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Microeconomics (mru.org)
+Khan Academy Microeconomics (khanacademy.org/economics-finance-domain/microeconomics)
+Freakonomics Radio Podcast (freakonomics.com)</t>
+        </is>
+      </c>
+      <c r="L13" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="A14" s="66" t="n"/>
+      <c r="B14" s="71" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="71" t="inlineStr">
         <is>
           <t>Microeconomics</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="71" t="inlineStr">
         <is>
           <t>MGTECON 209</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="71" t="inlineStr">
         <is>
           <t>Autumn</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="71" t="inlineStr">
         <is>
           <t>Analytical Foundations</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="G14" s="71" t="inlineStr">
         <is>
           <t>4 units</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="H14" s="71" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="I14" s="71" t="inlineStr">
         <is>
           <t>Microeconomics for managerial decision-making: markets, pricing, game theory, strategic interaction.</t>
         </is>
       </c>
-      <c r="J14" s="13" t="inlineStr">
+      <c r="J14" s="71" t="inlineStr">
         <is>
           <t>Micro</t>
         </is>
       </c>
+      <c r="K14" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Microeconomics (mru.org/courses/principles-of-microeconomics)
+Khan Academy Microeconomics (khanacademy.org/economics-finance-domain/microeconomics)</t>
+        </is>
+      </c>
+      <c r="L14" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="A15" s="66" t="n"/>
+      <c r="B15" s="71" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="71" t="inlineStr">
         <is>
           <t>Macroeconomics</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="71" t="inlineStr">
         <is>
           <t>MGTECON 240</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="71" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F15" s="71" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="G15" s="71" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="H15" s="71" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="I15" s="71" t="inlineStr">
         <is>
           <t>Macro environment: GDP, inflation, interest/exchange rates, monetary and fiscal policy.</t>
         </is>
       </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="J15" s="71" t="inlineStr">
         <is>
           <t>Macro</t>
         </is>
       </c>
+      <c r="K15" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Macroeconomics (mru.org/courses/principles-of-macroeconomics)
+Economics Explained (YT: youtube.com/c/EconomicsExplained)
+Khan Academy Macroeconomics (khanacademy.org/economics-finance-domain/macroeconomics)</t>
+        </is>
+      </c>
+      <c r="L15" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="A16" s="67" t="n"/>
+      <c r="B16" s="71" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="71" t="inlineStr">
         <is>
           <t>Strategy Beyond Markets</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="71" t="inlineStr">
         <is>
           <t>POLECON 239</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="71" t="inlineStr">
         <is>
           <t>Spring</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="71" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G16" s="71" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H16" s="71" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="I16" s="71" t="inlineStr">
         <is>
           <t>Political economy of business: lobbying, regulation, non-market strategy, business–government intersection.</t>
         </is>
       </c>
-      <c r="J16" s="13" t="inlineStr">
+      <c r="J16" s="71" t="inlineStr">
         <is>
           <t>Non-market / political economy</t>
         </is>
       </c>
+      <c r="K16" s="65" t="inlineStr">
+        <is>
+          <t>Freakonomics Radio – business &amp; political economy episodes (freakonomics.com)
+HBS Cold Call Podcast – ethics &amp; policy cases (hbr.org/2019/04/podcast-cold-call)
+HBR IdeaCast Podcast (hbr.org/podcasts)</t>
+        </is>
+      </c>
+      <c r="L16" s="65" t="inlineStr">
+        <is>
+          <t>— (no direct HBS Online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="72" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="73" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C17" s="73" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="73" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E17" s="73" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="73" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G17" s="73" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="H17" s="73" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
+      <c r="I17" s="73" t="inlineStr">
         <is>
           <t>Core frameworks: customer analysis, segmentation, targeting, positioning, the marketing mix.</t>
         </is>
       </c>
-      <c r="J17" s="16" t="inlineStr"/>
+      <c r="J17" s="73" t="inlineStr"/>
+      <c r="K17" s="65" t="inlineStr">
+        <is>
+          <t>HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
+Neil Patel – Digital Marketing Strategy (YT: youtube.com/neilpatel)
+Wharton Marketing on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="L17" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)
+Wharton Marketing on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="A18" s="66" t="n"/>
+      <c r="B18" s="73" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C18" s="73" t="inlineStr">
         <is>
           <t>Marketing Innovation</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="73" t="inlineStr">
         <is>
           <t>15.814</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="73" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F18" s="73" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G18" s="73" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="H18" s="73" t="inlineStr">
         <is>
           <t>Core Elective (choose 1 of 4)</t>
         </is>
       </c>
-      <c r="I18" s="16" t="inlineStr">
+      <c r="I18" s="73" t="inlineStr">
         <is>
           <t>Marketing strategy: consumer behavior, segmentation, positioning, product development, go-to-market.</t>
         </is>
       </c>
-      <c r="J18" s="16" t="inlineStr">
+      <c r="J18" s="73" t="inlineStr">
         <is>
           <t>One of 4 Sem-1 'core electives'</t>
         </is>
       </c>
+      <c r="K18" s="65" t="inlineStr">
+        <is>
+          <t>HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
+Neil Patel – Digital Marketing Strategy (YT: youtube.com/neilpatel)
+Wharton Marketing on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="L18" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="A19" s="67" t="n"/>
+      <c r="B19" s="73" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C19" s="16" t="inlineStr">
+      <c r="C19" s="73" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="73" t="inlineStr">
         <is>
           <t>MKTG 249</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="73" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F19" s="73" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G19" s="73" t="inlineStr">
         <is>
           <t>3–4 units</t>
         </is>
       </c>
-      <c r="H19" s="17" t="inlineStr">
+      <c r="H19" s="73" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I19" s="16" t="inlineStr">
+      <c r="I19" s="73" t="inlineStr">
         <is>
           <t>Marketing strategy: consumer behavior, segmentation, targeting, positioning, brand, marketing mix.</t>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr"/>
+      <c r="J19" s="73" t="inlineStr"/>
+      <c r="K19" s="65" t="inlineStr">
+        <is>
+          <t>HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
+Neil Patel – Digital Marketing Strategy (YT: youtube.com/neilpatel)</t>
+        </is>
+      </c>
+      <c r="L19" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)
+Wharton Marketing on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="74" t="inlineStr">
         <is>
           <t>Operations &amp; Technology Management</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B20" s="75" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="75" t="inlineStr">
         <is>
           <t>Technology and Operations Management (TOM)</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="75" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="75" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F20" s="19" t="inlineStr">
+      <c r="F20" s="75" t="inlineStr">
         <is>
           <t>Technology &amp; Operations</t>
         </is>
       </c>
-      <c r="G20" s="19" t="inlineStr">
+      <c r="G20" s="75" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H20" s="20" t="inlineStr">
+      <c r="H20" s="75" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I20" s="19" t="inlineStr">
+      <c r="I20" s="75" t="inlineStr">
         <is>
           <t>Process design, supply chain, quality management, and the role of technology in operations.</t>
         </is>
       </c>
-      <c r="J20" s="19" t="inlineStr"/>
+      <c r="J20" s="75" t="inlineStr"/>
+      <c r="K20" s="65" t="inlineStr">
+        <is>
+          <t>MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
+Wharton Operations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="L20" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)
+Wharton Operations on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="A21" s="66" t="n"/>
+      <c r="B21" s="75" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="75" t="inlineStr">
         <is>
           <t>Introduction to Operations Management</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="75" t="inlineStr">
         <is>
           <t>15.761</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="E21" s="75" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F21" s="19" t="inlineStr">
+      <c r="F21" s="75" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="G21" s="19" t="inlineStr">
+      <c r="G21" s="75" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H21" s="20" t="inlineStr">
+      <c r="H21" s="75" t="inlineStr">
         <is>
           <t>Core Elective (choose 1 of 4)</t>
         </is>
       </c>
-      <c r="I21" s="19" t="inlineStr">
+      <c r="I21" s="75" t="inlineStr">
         <is>
           <t>Process analysis, queuing, inventory, supply chain design, quality management.</t>
         </is>
       </c>
-      <c r="J21" s="19" t="inlineStr">
+      <c r="J21" s="75" t="inlineStr">
         <is>
           <t>One of 4 Sem-1 'core electives'</t>
         </is>
       </c>
+      <c r="K21" s="65" t="inlineStr">
+        <is>
+          <t>MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
+Wharton Operations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="L21" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)
+Wharton Operations on Coursera ~$49 cert</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n"/>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="A22" s="67" t="n"/>
+      <c r="B22" s="75" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="75" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="75" t="inlineStr">
         <is>
           <t>OIT 262</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="75" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="F22" s="19" t="inlineStr">
+      <c r="F22" s="75" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G22" s="19" t="inlineStr">
+      <c r="G22" s="75" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H22" s="20" t="inlineStr">
+      <c r="H22" s="75" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I22" s="19" t="inlineStr">
+      <c r="I22" s="75" t="inlineStr">
         <is>
           <t>Process analysis, capacity management, inventory, supply chains, quality fundamentals.</t>
         </is>
       </c>
-      <c r="J22" s="19" t="inlineStr"/>
+      <c r="J22" s="75" t="inlineStr"/>
+      <c r="K22" s="65" t="inlineStr">
+        <is>
+          <t>MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
+Wharton Operations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="L22" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="76" t="inlineStr">
         <is>
           <t>Data, Analytics, AI &amp; Information Systems</t>
         </is>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B23" s="77" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C23" s="22" t="inlineStr">
+      <c r="C23" s="77" t="inlineStr">
         <is>
           <t>Data Science and AI for Leaders (DSAIL)</t>
         </is>
       </c>
-      <c r="D23" s="22" t="inlineStr">
+      <c r="D23" s="77" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="22" t="inlineStr">
+      <c r="E23" s="77" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F23" s="22" t="inlineStr">
+      <c r="F23" s="77" t="inlineStr">
         <is>
           <t>Technology &amp; Analytics</t>
         </is>
       </c>
-      <c r="G23" s="22" t="inlineStr">
+      <c r="G23" s="77" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H23" s="23" t="inlineStr">
+      <c r="H23" s="77" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I23" s="22" t="inlineStr">
+      <c r="I23" s="77" t="inlineStr">
         <is>
           <t>AI tools, data-science fundamentals, applying AI to business decisions.</t>
         </is>
       </c>
-      <c r="J23" s="22" t="inlineStr">
+      <c r="J23" s="77" t="inlineStr">
         <is>
           <t>NEW (2025) – first AI-native required course at HBS; Class of 2027</t>
         </is>
       </c>
+      <c r="K23" s="65" t="inlineStr">
+        <is>
+          <t>Alex The Analyst – Full Data Analyst Bootcamp (YT: youtube.com/@AlexTheAnalyst)
+StatQuest with Josh Starmer – ML &amp; Stats (YT: youtube.com/c/joshstarmer)
+365 Data Science YouTube (youtube.com/c/365DataScience)</t>
+        </is>
+      </c>
+      <c r="L23" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)
+HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="A24" s="66" t="n"/>
+      <c r="B24" s="77" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C24" s="77" t="inlineStr">
         <is>
           <t>Data, Models and Decisions</t>
         </is>
       </c>
-      <c r="D24" s="22" t="inlineStr">
+      <c r="D24" s="77" t="inlineStr">
         <is>
           <t>15.060</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="77" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F24" s="22" t="inlineStr">
+      <c r="F24" s="77" t="inlineStr">
         <is>
           <t>Statistics / Analytics</t>
         </is>
       </c>
-      <c r="G24" s="22" t="inlineStr">
+      <c r="G24" s="77" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H24" s="23" t="inlineStr">
+      <c r="H24" s="77" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I24" s="22" t="inlineStr">
+      <c r="I24" s="77" t="inlineStr">
         <is>
           <t>Quantitative decision-making: probability, regression, simulation, optimization.</t>
         </is>
       </c>
-      <c r="J24" s="22" t="inlineStr"/>
+      <c r="J24" s="77" t="inlineStr"/>
+      <c r="K24" s="65" t="inlineStr">
+        <is>
+          <t>StatQuest with Josh Starmer – Statistics &amp; ML (YT: youtube.com/c/joshstarmer)
+Alex The Analyst (YT: youtube.com/@AlexTheAnalyst)
+Khan Academy Statistics &amp; Probability (khanacademy.org/math/statistics-probability)</t>
+        </is>
+      </c>
+      <c r="L24" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)
+HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="22" t="inlineStr">
+      <c r="A25" s="66" t="n"/>
+      <c r="B25" s="77" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C25" s="22" t="inlineStr">
+      <c r="C25" s="77" t="inlineStr">
         <is>
           <t>Data Analysis and Decision Making (Base / Accelerated)</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
+      <c r="D25" s="77" t="inlineStr">
         <is>
           <t>OB 358 / OB 360</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
+      <c r="E25" s="77" t="inlineStr">
         <is>
           <t>Autumn</t>
         </is>
       </c>
-      <c r="F25" s="22" t="inlineStr">
+      <c r="F25" s="77" t="inlineStr">
         <is>
           <t>Analytical Foundations</t>
         </is>
       </c>
-      <c r="G25" s="22" t="inlineStr">
+      <c r="G25" s="77" t="inlineStr">
         <is>
           <t>4 units</t>
         </is>
       </c>
-      <c r="H25" s="23" t="inlineStr">
+      <c r="H25" s="77" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I25" s="22" t="inlineStr">
+      <c r="I25" s="77" t="inlineStr">
         <is>
           <t>Probability, sampling, hypothesis testing, regression, basic ML prediction. Placed by assessment.</t>
         </is>
       </c>
-      <c r="J25" s="22" t="inlineStr">
+      <c r="J25" s="77" t="inlineStr">
         <is>
           <t>Base vs Accelerated track</t>
         </is>
       </c>
+      <c r="K25" s="65" t="inlineStr">
+        <is>
+          <t>StatQuest with Josh Starmer (YT: youtube.com/c/joshstarmer)
+Alex The Analyst (YT: youtube.com/@AlexTheAnalyst)
+Khan Academy Statistics (khanacademy.org/math/statistics-probability)</t>
+        </is>
+      </c>
+      <c r="L25" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="A26" s="66" t="n"/>
+      <c r="B26" s="77" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C26" s="22" t="inlineStr">
+      <c r="C26" s="77" t="inlineStr">
         <is>
           <t>Optimization and Simulation Modeling</t>
         </is>
       </c>
-      <c r="D26" s="22" t="inlineStr">
+      <c r="D26" s="77" t="inlineStr">
         <is>
           <t>MS&amp;E 348</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
+      <c r="E26" s="77" t="inlineStr">
         <is>
           <t>Autumn</t>
         </is>
       </c>
-      <c r="F26" s="22" t="inlineStr">
+      <c r="F26" s="77" t="inlineStr">
         <is>
           <t>Analytical Foundations</t>
         </is>
       </c>
-      <c r="G26" s="22" t="inlineStr">
+      <c r="G26" s="77" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H26" s="23" t="inlineStr">
+      <c r="H26" s="77" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I26" s="22" t="inlineStr">
+      <c r="I26" s="77" t="inlineStr">
         <is>
           <t>Linear/integer programming, simulation, decision analysis for business optimization.</t>
         </is>
       </c>
-      <c r="J26" s="22" t="inlineStr"/>
+      <c r="J26" s="77" t="inlineStr"/>
+      <c r="K26" s="65" t="inlineStr">
+        <is>
+          <t>StatQuest with Josh Starmer – ML/optimization concepts (YT: youtube.com/c/joshstarmer)
+365 Data Science (YT: youtube.com/c/365DataScience)</t>
+        </is>
+      </c>
+      <c r="L26" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n"/>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="A27" s="67" t="n"/>
+      <c r="B27" s="77" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C27" s="22" t="inlineStr">
+      <c r="C27" s="77" t="inlineStr">
         <is>
           <t>Information Management</t>
         </is>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D27" s="77" t="inlineStr">
         <is>
           <t>OIT 335</t>
         </is>
       </c>
-      <c r="E27" s="22" t="inlineStr">
+      <c r="E27" s="77" t="inlineStr">
         <is>
           <t>Spring</t>
         </is>
       </c>
-      <c r="F27" s="22" t="inlineStr">
+      <c r="F27" s="77" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G27" s="22" t="inlineStr">
+      <c r="G27" s="77" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H27" s="23" t="inlineStr">
+      <c r="H27" s="77" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I27" s="22" t="inlineStr">
+      <c r="I27" s="77" t="inlineStr">
         <is>
           <t>IT strategy, digital platforms, data management, role of information systems in business.</t>
         </is>
       </c>
-      <c r="J27" s="22" t="inlineStr"/>
+      <c r="J27" s="77" t="inlineStr"/>
+      <c r="K27" s="65" t="inlineStr">
+        <is>
+          <t>HBR IdeaCast – Digital transformation episodes (hbr.org/podcasts)
+Stanford GSB YouTube – technology strategy talks (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
+        </is>
+      </c>
+      <c r="L27" s="65" t="inlineStr">
+        <is>
+          <t>— (no direct HBS Online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="78" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="B28" s="25" t="inlineStr">
+      <c r="B28" s="79" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C28" s="25" t="inlineStr">
+      <c r="C28" s="79" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="D28" s="25" t="inlineStr">
+      <c r="D28" s="79" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="25" t="inlineStr">
+      <c r="E28" s="79" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F28" s="25" t="inlineStr">
+      <c r="F28" s="79" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="G28" s="25" t="inlineStr">
+      <c r="G28" s="79" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H28" s="26" t="inlineStr">
+      <c r="H28" s="79" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I28" s="25" t="inlineStr">
+      <c r="I28" s="79" t="inlineStr">
         <is>
           <t>Competitive strategy frameworks: industry analysis, competitive advantage, positioning.</t>
         </is>
       </c>
-      <c r="J28" s="25" t="inlineStr"/>
+      <c r="J28" s="79" t="inlineStr"/>
+      <c r="K28" s="65" t="inlineStr">
+        <is>
+          <t>Modern MBA – case-method strategy deep dives (YT: youtube.com/c/ModernMBA)
+Acquired Podcast – company strategy histories (acquired.fm)
+HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)
+Stanford GSB YouTube (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
+        </is>
+      </c>
+      <c r="L28" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)
+HBS Online Core Business Essentials ~$2,650 – includes Strategy module (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="25" t="inlineStr">
+      <c r="A29" s="66" t="n"/>
+      <c r="B29" s="79" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C29" s="25" t="inlineStr">
+      <c r="C29" s="79" t="inlineStr">
         <is>
           <t>Competitive Strategy</t>
         </is>
       </c>
-      <c r="D29" s="25" t="inlineStr">
+      <c r="D29" s="79" t="inlineStr">
         <is>
           <t>15.900</t>
         </is>
       </c>
-      <c r="E29" s="25" t="inlineStr">
+      <c r="E29" s="79" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F29" s="25" t="inlineStr">
+      <c r="F29" s="79" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="G29" s="25" t="inlineStr">
+      <c r="G29" s="79" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H29" s="26" t="inlineStr">
+      <c r="H29" s="79" t="inlineStr">
         <is>
           <t>Core Elective (choose 1 of 4)</t>
         </is>
       </c>
-      <c r="I29" s="25" t="inlineStr">
+      <c r="I29" s="79" t="inlineStr">
         <is>
           <t>Industry analysis, competitive positioning, strategic planning, dynamic strategy.</t>
         </is>
       </c>
-      <c r="J29" s="25" t="inlineStr">
+      <c r="J29" s="79" t="inlineStr">
         <is>
           <t>One of 4 Sem-1 'core electives'</t>
         </is>
       </c>
+      <c r="K29" s="65" t="inlineStr">
+        <is>
+          <t>Modern MBA (YT: youtube.com/c/ModernMBA)
+Acquired Podcast (acquired.fm)
+HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)</t>
+        </is>
+      </c>
+      <c r="L29" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)
+Wharton Business Foundations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="n"/>
-      <c r="B30" s="25" t="inlineStr">
+      <c r="A30" s="67" t="n"/>
+      <c r="B30" s="79" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
+      <c r="C30" s="79" t="inlineStr">
         <is>
           <t>Strategic Leadership</t>
         </is>
       </c>
-      <c r="D30" s="25" t="inlineStr">
+      <c r="D30" s="79" t="inlineStr">
         <is>
           <t>STRAMGT 259</t>
         </is>
       </c>
-      <c r="E30" s="25" t="inlineStr">
+      <c r="E30" s="79" t="inlineStr">
         <is>
           <t>Spring</t>
         </is>
       </c>
-      <c r="F30" s="25" t="inlineStr">
+      <c r="F30" s="79" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G30" s="25" t="inlineStr">
+      <c r="G30" s="79" t="inlineStr">
         <is>
           <t>3–4 units</t>
         </is>
       </c>
-      <c r="H30" s="26" t="inlineStr">
+      <c r="H30" s="79" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I30" s="25" t="inlineStr">
+      <c r="I30" s="79" t="inlineStr">
         <is>
           <t>Integrative: competitive strategy, industry analysis, leadership in executing strategy. Bridge to Year 2.</t>
         </is>
       </c>
-      <c r="J30" s="25" t="inlineStr"/>
+      <c r="J30" s="79" t="inlineStr"/>
+      <c r="K30" s="65" t="inlineStr">
+        <is>
+          <t>Modern MBA (YT: youtube.com/c/ModernMBA)
+Stanford GSB YouTube – strategy talks (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)
+HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)</t>
+        </is>
+      </c>
+      <c r="L30" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="inlineStr">
+      <c r="A31" s="80" t="inlineStr">
         <is>
           <t>Organizational Behavior, Leadership &amp; People</t>
         </is>
       </c>
-      <c r="B31" s="28" t="inlineStr">
+      <c r="B31" s="81" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C31" s="28" t="inlineStr">
+      <c r="C31" s="81" t="inlineStr">
         <is>
           <t>Leadership and Organizational Behavior (LEAD)</t>
         </is>
       </c>
-      <c r="D31" s="28" t="inlineStr">
+      <c r="D31" s="81" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E31" s="28" t="inlineStr">
+      <c r="E31" s="81" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F31" s="28" t="inlineStr">
+      <c r="F31" s="81" t="inlineStr">
         <is>
           <t>Organizational Behavior</t>
         </is>
       </c>
-      <c r="G31" s="28" t="inlineStr">
+      <c r="G31" s="81" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H31" s="29" t="inlineStr">
+      <c r="H31" s="81" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I31" s="28" t="inlineStr">
+      <c r="I31" s="81" t="inlineStr">
         <is>
           <t>Individual/group behavior: motivation, team dynamics, leadership styles, organizational culture.</t>
         </is>
       </c>
-      <c r="J31" s="28" t="inlineStr"/>
+      <c r="J31" s="81" t="inlineStr"/>
+      <c r="K31" s="65" t="inlineStr">
+        <is>
+          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)
+Stanford GSB YouTube (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)
+HBR IdeaCast Podcast (hbr.org/podcasts)
+TED Business (YT: youtube.com/c/TEDBusiness)</t>
+        </is>
+      </c>
+      <c r="L31" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)
+HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="n"/>
-      <c r="B32" s="28" t="inlineStr">
+      <c r="A32" s="66" t="n"/>
+      <c r="B32" s="81" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C32" s="28" t="inlineStr">
+      <c r="C32" s="81" t="inlineStr">
         <is>
           <t>Organizational Processes</t>
         </is>
       </c>
-      <c r="D32" s="28" t="inlineStr">
+      <c r="D32" s="81" t="inlineStr">
         <is>
           <t>15.311</t>
         </is>
       </c>
-      <c r="E32" s="28" t="inlineStr">
+      <c r="E32" s="81" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F32" s="28" t="inlineStr">
+      <c r="F32" s="81" t="inlineStr">
         <is>
           <t>Org Behavior / Management</t>
         </is>
       </c>
-      <c r="G32" s="28" t="inlineStr">
+      <c r="G32" s="81" t="inlineStr">
         <is>
           <t>9 units</t>
         </is>
       </c>
-      <c r="H32" s="29" t="inlineStr">
+      <c r="H32" s="81" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I32" s="28" t="inlineStr">
+      <c r="I32" s="81" t="inlineStr">
         <is>
           <t>How organizations function: decision-making, culture, change management, leadership, human capital.</t>
         </is>
       </c>
-      <c r="J32" s="28" t="inlineStr"/>
+      <c r="J32" s="81" t="inlineStr"/>
+      <c r="K32" s="65" t="inlineStr">
+        <is>
+          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)
+HBR IdeaCast Podcast (hbr.org/podcasts)</t>
+        </is>
+      </c>
+      <c r="L32" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)
+HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="28" t="inlineStr">
+      <c r="A33" s="66" t="n"/>
+      <c r="B33" s="81" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C33" s="28" t="inlineStr">
+      <c r="C33" s="81" t="inlineStr">
         <is>
           <t>Organizational Behavior / Managing Groups and Teams</t>
         </is>
       </c>
-      <c r="D33" s="28" t="inlineStr">
+      <c r="D33" s="81" t="inlineStr">
         <is>
           <t>OB 270 / GSBGEN 566</t>
         </is>
       </c>
-      <c r="E33" s="28" t="inlineStr">
+      <c r="E33" s="81" t="inlineStr">
         <is>
           <t>Autumn</t>
         </is>
       </c>
-      <c r="F33" s="28" t="inlineStr">
+      <c r="F33" s="81" t="inlineStr">
         <is>
           <t>Leadership Foundations</t>
         </is>
       </c>
-      <c r="G33" s="28" t="inlineStr">
+      <c r="G33" s="81" t="inlineStr">
         <is>
           <t>3–4 units</t>
         </is>
       </c>
-      <c r="H33" s="29" t="inlineStr">
+      <c r="H33" s="81" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I33" s="28" t="inlineStr">
+      <c r="I33" s="81" t="inlineStr">
         <is>
           <t>Behavioral foundations: motivation, team dynamics, leadership, culture; team performance &amp; group decisions.</t>
         </is>
       </c>
-      <c r="J33" s="28" t="inlineStr"/>
+      <c r="J33" s="81" t="inlineStr"/>
+      <c r="K33" s="65" t="inlineStr">
+        <is>
+          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)
+Stanford GSB YouTube (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)
+TED Business (YT: youtube.com/c/TEDBusiness)</t>
+        </is>
+      </c>
+      <c r="L33" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="n"/>
-      <c r="B34" s="28" t="inlineStr">
+      <c r="A34" s="67" t="n"/>
+      <c r="B34" s="81" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C34" s="28" t="inlineStr">
+      <c r="C34" s="81" t="inlineStr">
         <is>
           <t>Human Resource Management</t>
         </is>
       </c>
-      <c r="D34" s="28" t="inlineStr">
+      <c r="D34" s="81" t="inlineStr">
         <is>
           <t>GSBGEN 518</t>
         </is>
       </c>
-      <c r="E34" s="28" t="inlineStr">
+      <c r="E34" s="81" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="F34" s="28" t="inlineStr">
+      <c r="F34" s="81" t="inlineStr">
         <is>
           <t>Management Foundations</t>
         </is>
       </c>
-      <c r="G34" s="28" t="inlineStr">
+      <c r="G34" s="81" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H34" s="29" t="inlineStr">
+      <c r="H34" s="81" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I34" s="28" t="inlineStr">
+      <c r="I34" s="81" t="inlineStr">
         <is>
           <t>Talent acquisition, performance management, compensation, org design, HR strategy.</t>
         </is>
       </c>
-      <c r="J34" s="28" t="inlineStr"/>
+      <c r="J34" s="81" t="inlineStr"/>
+      <c r="K34" s="65" t="inlineStr">
+        <is>
+          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+HBR IdeaCast Podcast – people &amp; talent episodes (hbr.org/podcasts)</t>
+        </is>
+      </c>
+      <c r="L34" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="30" t="inlineStr">
+      <c r="A35" s="82" t="inlineStr">
         <is>
           <t>Ethics, Accountability &amp; Social Purpose</t>
         </is>
       </c>
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="83" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C35" s="31" t="inlineStr">
+      <c r="C35" s="83" t="inlineStr">
         <is>
           <t>Leadership and Corporate Accountability (LCA)</t>
         </is>
       </c>
-      <c r="D35" s="31" t="inlineStr">
+      <c r="D35" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E35" s="31" t="inlineStr">
+      <c r="E35" s="83" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F35" s="31" t="inlineStr">
+      <c r="F35" s="83" t="inlineStr">
         <is>
           <t>Ethics &amp; Leadership</t>
         </is>
       </c>
-      <c r="G35" s="31" t="inlineStr">
+      <c r="G35" s="83" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H35" s="32" t="inlineStr">
+      <c r="H35" s="83" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I35" s="31" t="inlineStr">
+      <c r="I35" s="83" t="inlineStr">
         <is>
           <t>Ethical decision-making, corporate responsibility, stakeholder management, legal dimensions of leadership.</t>
         </is>
       </c>
-      <c r="J35" s="31" t="inlineStr"/>
+      <c r="J35" s="83" t="inlineStr"/>
+      <c r="K35" s="65" t="inlineStr">
+        <is>
+          <t>HBS Cold Call Podcast – ethics cases (hbr.org/2019/04/podcast-cold-call)
+Edspira – Business Ethics module (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)
+HBR IdeaCast Podcast (hbr.org/podcasts)</t>
+        </is>
+      </c>
+      <c r="L35" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Negotiation Mastery ~$1,850 (online.hbs.edu/courses/negotiation)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="31" t="inlineStr">
+      <c r="A36" s="66" t="n"/>
+      <c r="B36" s="83" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C36" s="31" t="inlineStr">
+      <c r="C36" s="83" t="inlineStr">
         <is>
           <t>Inclusion and Social Purpose of the Firm (SPF)</t>
         </is>
       </c>
-      <c r="D36" s="31" t="inlineStr">
+      <c r="D36" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E36" s="31" t="inlineStr">
+      <c r="E36" s="83" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F36" s="31" t="inlineStr">
+      <c r="F36" s="83" t="inlineStr">
         <is>
           <t>General Management / Ethics</t>
         </is>
       </c>
-      <c r="G36" s="31" t="inlineStr">
+      <c r="G36" s="83" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H36" s="32" t="inlineStr">
+      <c r="H36" s="83" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I36" s="31" t="inlineStr">
+      <c r="I36" s="83" t="inlineStr">
         <is>
           <t>Two modules: diversity &amp; inclusion in the workplace + the firm's responsibility to society.</t>
         </is>
       </c>
-      <c r="J36" s="31" t="inlineStr">
+      <c r="J36" s="83" t="inlineStr">
         <is>
           <t>Two-module course</t>
         </is>
       </c>
+      <c r="K36" s="65" t="inlineStr">
+        <is>
+          <t>HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)
+HBR IdeaCast – CSR &amp; social purpose episodes (hbr.org/podcasts)
+TED Business – ethics talks (YT: youtube.com/c/TEDBusiness)</t>
+        </is>
+      </c>
+      <c r="L36" s="65" t="inlineStr">
+        <is>
+          <t>— (no direct HBS Online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n"/>
-      <c r="B37" s="31" t="inlineStr">
+      <c r="A37" s="67" t="n"/>
+      <c r="B37" s="83" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C37" s="31" t="inlineStr">
+      <c r="C37" s="83" t="inlineStr">
         <is>
           <t>Leading with Values (Ethics)</t>
         </is>
       </c>
-      <c r="D37" s="31" t="inlineStr">
+      <c r="D37" s="83" t="inlineStr">
         <is>
           <t>GSBGEN 567</t>
         </is>
       </c>
-      <c r="E37" s="31" t="inlineStr">
+      <c r="E37" s="83" t="inlineStr">
         <is>
           <t>Autumn</t>
         </is>
       </c>
-      <c r="F37" s="31" t="inlineStr">
+      <c r="F37" s="83" t="inlineStr">
         <is>
           <t>Leadership Foundations</t>
         </is>
       </c>
-      <c r="G37" s="31" t="inlineStr">
+      <c r="G37" s="83" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H37" s="32" t="inlineStr">
+      <c r="H37" s="83" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I37" s="31" t="inlineStr">
+      <c r="I37" s="83" t="inlineStr">
         <is>
           <t>Ethical reasoning; frameworks for moral dilemmas; corporate responsibility; values-based leadership.</t>
         </is>
       </c>
-      <c r="J37" s="31" t="inlineStr"/>
+      <c r="J37" s="83" t="inlineStr"/>
+      <c r="K37" s="65" t="inlineStr">
+        <is>
+          <t>HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)
+TED Business (YT: youtube.com/c/TEDBusiness)
+HBR IdeaCast Podcast (hbr.org/podcasts)</t>
+        </is>
+      </c>
+      <c r="L37" s="65" t="inlineStr">
+        <is>
+          <t>— (no direct HBS Online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="33" t="inlineStr">
+      <c r="A38" s="84" t="inlineStr">
         <is>
           <t>Entrepreneurship</t>
         </is>
       </c>
-      <c r="B38" s="34" t="inlineStr">
+      <c r="B38" s="85" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C38" s="34" t="inlineStr">
+      <c r="C38" s="85" t="inlineStr">
         <is>
           <t>The Entrepreneurial Manager (TEM)</t>
         </is>
       </c>
-      <c r="D38" s="34" t="inlineStr">
+      <c r="D38" s="85" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="34" t="inlineStr">
+      <c r="E38" s="85" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F38" s="34" t="inlineStr">
+      <c r="F38" s="85" t="inlineStr">
         <is>
           <t>Entrepreneurial Management</t>
         </is>
       </c>
-      <c r="G38" s="34" t="inlineStr">
+      <c r="G38" s="85" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H38" s="35" t="inlineStr">
+      <c r="H38" s="85" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I38" s="34" t="inlineStr">
+      <c r="I38" s="85" t="inlineStr">
         <is>
           <t>Entrepreneurial thinking for new ventures and within firms; opportunity recognition, resource acquisition.</t>
         </is>
       </c>
-      <c r="J38" s="34" t="inlineStr">
+      <c r="J38" s="85" t="inlineStr">
         <is>
           <t>Only school with required Y1 entrepreneurship</t>
         </is>
       </c>
+      <c r="K38" s="65" t="inlineStr">
+        <is>
+          <t>Y Combinator Startup School (YT: youtube.com/@ycombinator; startupschool.org/curriculum)
+Stanford eCorner – 2,000+ entrepreneur videos (ecorner.stanford.edu)
+HBS Cold Call Podcast – entrepreneurship episodes (hbr.org/2019/04/podcast-cold-call)</t>
+        </is>
+      </c>
+      <c r="L38" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Entrepreneurship Essentials ~$1,850 (online.hbs.edu/courses/entrepreneurship-essentials)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="36" t="inlineStr">
+      <c r="A39" s="86" t="inlineStr">
         <is>
           <t>Business Communication</t>
         </is>
       </c>
-      <c r="B39" s="37" t="inlineStr">
+      <c r="B39" s="87" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C39" s="37" t="inlineStr">
+      <c r="C39" s="87" t="inlineStr">
         <is>
           <t>Communication for Leaders</t>
         </is>
       </c>
-      <c r="D39" s="37" t="inlineStr">
+      <c r="D39" s="87" t="inlineStr">
         <is>
           <t>15.280</t>
         </is>
       </c>
-      <c r="E39" s="37" t="inlineStr">
+      <c r="E39" s="87" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F39" s="37" t="inlineStr">
+      <c r="F39" s="87" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="G39" s="37" t="inlineStr">
+      <c r="G39" s="87" t="inlineStr">
         <is>
           <t>6 units</t>
         </is>
       </c>
-      <c r="H39" s="38" t="inlineStr">
+      <c r="H39" s="87" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I39" s="37" t="inlineStr">
+      <c r="I39" s="87" t="inlineStr">
         <is>
           <t>Written &amp; oral business communication: structuring arguments, presentations, memos, difficult conversations.</t>
         </is>
       </c>
-      <c r="J39" s="37" t="inlineStr">
+      <c r="J39" s="87" t="inlineStr">
         <is>
           <t>Only school with required Y1 communication</t>
         </is>
       </c>
+      <c r="K39" s="65" t="inlineStr">
+        <is>
+          <t>TED Business – communication &amp; presentation talks (YT: youtube.com/c/TEDBusiness)
+Stanford GSB YouTube – communication &amp; public speaking (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
+        </is>
+      </c>
+      <c r="L39" s="65" t="inlineStr">
+        <is>
+          <t>— (no direct HBS Online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="39" t="inlineStr">
+      <c r="A40" s="88" t="inlineStr">
         <is>
           <t>Experiential &amp; Global Immersion</t>
         </is>
       </c>
-      <c r="B40" s="40" t="inlineStr">
+      <c r="B40" s="89" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C40" s="40" t="inlineStr">
+      <c r="C40" s="89" t="inlineStr">
         <is>
           <t>FIELD Foundations (FIELD 1)</t>
         </is>
       </c>
-      <c r="D40" s="40" t="inlineStr">
+      <c r="D40" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E40" s="40" t="inlineStr">
+      <c r="E40" s="89" t="inlineStr">
         <is>
           <t>Term 1 (Fall)</t>
         </is>
       </c>
-      <c r="F40" s="40" t="inlineStr">
+      <c r="F40" s="89" t="inlineStr">
         <is>
           <t>Experiential / Leadership</t>
         </is>
       </c>
-      <c r="G40" s="40" t="inlineStr">
+      <c r="G40" s="89" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H40" s="41" t="inlineStr">
+      <c r="H40" s="89" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I40" s="40" t="inlineStr">
+      <c r="I40" s="89" t="inlineStr">
         <is>
           <t>Leadership development workshops, self-assessment, team exercises; preps for the Global Capstone.</t>
         </is>
       </c>
-      <c r="J40" s="40" t="inlineStr">
+      <c r="J40" s="89" t="inlineStr">
         <is>
           <t>FIELD program</t>
         </is>
       </c>
+      <c r="K40" s="65" t="inlineStr">
+        <is>
+          <t>— (experiential program; no direct online equivalent)</t>
+        </is>
+      </c>
+      <c r="L40" s="65" t="inlineStr">
+        <is>
+          <t>— (experiential program; no direct online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="n"/>
-      <c r="B41" s="40" t="inlineStr">
+      <c r="A41" s="66" t="n"/>
+      <c r="B41" s="89" t="inlineStr">
         <is>
           <t>HBS</t>
         </is>
       </c>
-      <c r="C41" s="40" t="inlineStr">
+      <c r="C41" s="89" t="inlineStr">
         <is>
           <t>FIELD Global Capstone (FIELD 2)</t>
         </is>
       </c>
-      <c r="D41" s="40" t="inlineStr">
+      <c r="D41" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E41" s="40" t="inlineStr">
+      <c r="E41" s="89" t="inlineStr">
         <is>
           <t>Term 2 (Spring)</t>
         </is>
       </c>
-      <c r="F41" s="40" t="inlineStr">
+      <c r="F41" s="89" t="inlineStr">
         <is>
           <t>Experiential / Global</t>
         </is>
       </c>
-      <c r="G41" s="40" t="inlineStr">
+      <c r="G41" s="89" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="H41" s="41" t="inlineStr">
+      <c r="H41" s="89" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I41" s="40" t="inlineStr">
+      <c r="I41" s="89" t="inlineStr">
         <is>
           <t>Teams partner with a global company to build a product/service; 6–14 day international immersion.</t>
         </is>
       </c>
-      <c r="J41" s="40" t="inlineStr">
+      <c r="J41" s="89" t="inlineStr">
         <is>
           <t>Destinations incl. Ghana, Japan, Saudi Arabia, India, etc.</t>
         </is>
       </c>
+      <c r="K41" s="65" t="inlineStr">
+        <is>
+          <t>— (experiential / global immersion; no direct online equivalent)</t>
+        </is>
+      </c>
+      <c r="L41" s="65" t="inlineStr">
+        <is>
+          <t>— (experiential / global immersion; no direct online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n"/>
-      <c r="B42" s="40" t="inlineStr">
+      <c r="A42" s="66" t="n"/>
+      <c r="B42" s="89" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
         </is>
       </c>
-      <c r="C42" s="40" t="inlineStr">
+      <c r="C42" s="89" t="inlineStr">
         <is>
           <t>Leadership Challenges for an Inclusive World (LEAD Week)</t>
         </is>
       </c>
-      <c r="D42" s="40" t="inlineStr">
+      <c r="D42" s="89" t="inlineStr">
         <is>
           <t>15.002</t>
         </is>
       </c>
-      <c r="E42" s="40" t="inlineStr">
+      <c r="E42" s="89" t="inlineStr">
         <is>
           <t>Fall (Sem 1)</t>
         </is>
       </c>
-      <c r="F42" s="40" t="inlineStr">
+      <c r="F42" s="89" t="inlineStr">
         <is>
           <t>Leadership / Inclusion</t>
         </is>
       </c>
-      <c r="G42" s="40" t="inlineStr">
+      <c r="G42" s="89" t="inlineStr">
         <is>
           <t>3 units</t>
         </is>
       </c>
-      <c r="H42" s="41" t="inlineStr">
+      <c r="H42" s="89" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I42" s="40" t="inlineStr">
+      <c r="I42" s="89" t="inlineStr">
         <is>
           <t>3-day immersive off-campus experience; workshops on leadership values, inclusive practices, integrity.</t>
         </is>
       </c>
-      <c r="J42" s="40" t="inlineStr">
+      <c r="J42" s="89" t="inlineStr">
         <is>
           <t>Mid-October; also inclusion-focused</t>
         </is>
       </c>
+      <c r="K42" s="65" t="inlineStr">
+        <is>
+          <t>HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)</t>
+        </is>
+      </c>
+      <c r="L42" s="65" t="inlineStr">
+        <is>
+          <t>— (immersive off-campus; no direct online equivalent)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="n"/>
-      <c r="B43" s="40" t="inlineStr">
+      <c r="A43" s="66" t="n"/>
+      <c r="B43" s="89" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C43" s="40" t="inlineStr">
+      <c r="C43" s="89" t="inlineStr">
         <is>
           <t>Leadership Labs</t>
         </is>
       </c>
-      <c r="D43" s="40" t="inlineStr">
+      <c r="D43" s="89" t="inlineStr">
         <is>
           <t>GSBGEN</t>
         </is>
       </c>
-      <c r="E43" s="40" t="inlineStr">
+      <c r="E43" s="89" t="inlineStr">
         <is>
           <t>Autumn (Year 1)</t>
         </is>
       </c>
-      <c r="F43" s="40" t="inlineStr">
+      <c r="F43" s="89" t="inlineStr">
         <is>
           <t>Leadership Foundations</t>
         </is>
       </c>
-      <c r="G43" s="40" t="inlineStr">
+      <c r="G43" s="89" t="inlineStr">
         <is>
           <t>Non-credit / 1 unit</t>
         </is>
       </c>
-      <c r="H43" s="41" t="inlineStr">
+      <c r="H43" s="89" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I43" s="40" t="inlineStr">
+      <c r="I43" s="89" t="inlineStr">
         <is>
           <t>Small-group experiential workshops on self-awareness, interpersonal effectiveness, leadership style.</t>
         </is>
       </c>
-      <c r="J43" s="40" t="inlineStr">
+      <c r="J43" s="89" t="inlineStr">
         <is>
           <t>Coach-facilitated throughout Year 1</t>
         </is>
       </c>
+      <c r="K43" s="65" t="inlineStr">
+        <is>
+          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+Stanford GSB YouTube (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
+        </is>
+      </c>
+      <c r="L43" s="65" t="inlineStr">
+        <is>
+          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="n"/>
-      <c r="B44" s="40" t="inlineStr">
+      <c r="A44" s="67" t="n"/>
+      <c r="B44" s="89" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
         </is>
       </c>
-      <c r="C44" s="40" t="inlineStr">
+      <c r="C44" s="89" t="inlineStr">
         <is>
           <t>Global Experience Requirement (GER)</t>
         </is>
       </c>
-      <c r="D44" s="40" t="inlineStr">
+      <c r="D44" s="89" t="inlineStr">
         <is>
           <t>GSBGEN 580+</t>
         </is>
       </c>
-      <c r="E44" s="40" t="inlineStr">
+      <c r="E44" s="89" t="inlineStr">
         <is>
           <t>Year 1 (any quarter)</t>
         </is>
       </c>
-      <c r="F44" s="40" t="inlineStr">
+      <c r="F44" s="89" t="inlineStr">
         <is>
           <t>Global Experience</t>
         </is>
       </c>
-      <c r="G44" s="40" t="inlineStr">
+      <c r="G44" s="89" t="inlineStr">
         <is>
           <t>Varies</t>
         </is>
       </c>
-      <c r="H44" s="41" t="inlineStr">
+      <c r="H44" s="89" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="I44" s="40" t="inlineStr">
+      <c r="I44" s="89" t="inlineStr">
         <is>
           <t>Choose one: GMIX (4-wk immersion in 90+ countries), Global Seminars, Global Study Trips, STEP (Tsinghua), or Self-Directed Global Project.</t>
         </is>
       </c>
-      <c r="J44" s="40" t="inlineStr">
+      <c r="J44" s="89" t="inlineStr">
         <is>
           <t>Required global component</t>
+        </is>
+      </c>
+      <c r="K44" s="65" t="inlineStr">
+        <is>
+          <t>— (global immersion requirement; no direct online equivalent)</t>
+        </is>
+      </c>
+      <c r="L44" s="65" t="inlineStr">
+        <is>
+          <t>— (global immersion requirement; no direct online equivalent)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A40:A44"/>
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A4:A7"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A35:A37"/>
     <mergeCell ref="A12:A16"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="A40:A44"/>
     <mergeCell ref="A8:A11"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="A31:A34"/>
@@ -2789,7 +3394,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>Topic Coverage Matrix — which schools teach each topic in Year 1</t>
+          <t>Topic Coverage Matrix — which schools teach each topic in Year 1  | Free &amp; paid learning resources added to Master sheet (cols K–L)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Stanford GSB-specific official resources to all 17 Stanford course rows
Prepended Stanford-official resources (★ STANFORD OFFICIAL section) to the
Free and Paid resource columns for all 17 Stanford GSB first-year courses,
covering: GSB YouTube playlists (View From The Top, Class Takeaways), 4 GSB
podcasts (Think Fast Talk Smart, View From Top, If/Then, All Else Equal),
publicly available syllabi PDFs (Pfeffer OB 377, Admati FINANCE 332,
POLECON 239), Stanford Online paid courses (LEAD, Paths to Power, MS&E 240/
276/280), Coursera free-audit courses (Org Analysis, Game Theory), edX
Principles of Economics, eCorner ETL series, SSIR, and GSB exec-ed programs.

https://claude.ai/code/session_011QHxcNSM1P2957ocCew2SU
</commit_message>
<xml_diff>
--- a/m7_year1_master_by_topic.xlsx
+++ b/m7_year1_master_by_topic.xlsx
@@ -991,7 +991,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="66" t="n"/>
+      <c r="A5" s="7" t="n"/>
       <c r="B5" s="64" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -1048,7 +1048,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="66" t="n"/>
+      <c r="A6" s="7" t="n"/>
       <c r="B6" s="64" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1092,20 +1092,28 @@
       <c r="J6" s="64" t="inlineStr"/>
       <c r="K6" s="65" t="inlineStr">
         <is>
-          <t>Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Class Takeaways – Accounting Literacy (Prof. Ed deHaan) [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+ACCT 210 Syllabus 2019 (studocu.com/en-us/document/stanford-university/financial-accounting/acct-210-syllabus-2019/7696528)
+Stanford GSB Case Studies – free cases (gsb.stanford.edu/faculty-research/case-studies)
+★ GENERAL:
+Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
 MIT OCW Financial Accounting 15.515 (ocw.mit.edu/courses/15-515-financial-accounting-fall-2003/)
 Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)</t>
         </is>
       </c>
       <c r="L6" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+          <t>★ STANFORD OFFICIAL:
+Stanford Online MS&amp;E 240 Accounting for Managers &amp; Entrepreneurs (online.stanford.edu/courses/mse240-accounting-managers-and-entrepreneurs)
+★ OTHER PAID:
+HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="67" t="n"/>
+      <c r="A7" s="8" t="n"/>
       <c r="B7" s="64" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1149,14 +1157,21 @@
       <c r="J7" s="64" t="inlineStr"/>
       <c r="K7" s="65" t="inlineStr">
         <is>
-          <t>Edspira – Managerial Accounting series (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Class Takeaways – Accounting Literacy (Prof. Ed deHaan) [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+Stanford GSB Case Studies – free cases (gsb.stanford.edu/faculty-research/case-studies)
+★ GENERAL:
+Edspira – Managerial Accounting series (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
 Farhat Accounting Lectures – Managerial Accounting (YT: search 'Farhat Lectures')
 Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)</t>
         </is>
       </c>
       <c r="L7" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+          <t>★ STANFORD OFFICIAL:
+Stanford Online MS&amp;E 240 Accounting for Managers &amp; Entrepreneurs (online.stanford.edu/courses/mse240-accounting-managers-and-entrepreneurs)
+★ OTHER PAID:
+HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
@@ -1224,7 +1239,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="66" t="n"/>
+      <c r="A9" s="7" t="n"/>
       <c r="B9" s="69" t="inlineStr">
         <is>
           <t>HBS</t>
@@ -1280,7 +1295,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="66" t="n"/>
+      <c r="A10" s="7" t="n"/>
       <c r="B10" s="69" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -1341,7 +1356,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="67" t="n"/>
+      <c r="A11" s="8" t="n"/>
       <c r="B11" s="69" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1385,14 +1400,23 @@
       <c r="J11" s="69" t="inlineStr"/>
       <c r="K11" s="65" t="inlineStr">
         <is>
-          <t>Aswath Damodaran – Valuation MBA Spring 2025 (YT: youtube.com/playlist?list=PLUkh9m2BorqkgpNyRpP-NL3BS4yvFabXk)
+          <t>★ STANFORD OFFICIAL:
+Anat Admati – FINANCE 332 Syllabus PDF (gsb-faculty.stanford.edu/anat-r-admati)
+All Else Equal Podcast – finance &amp; decision-making (gsb.stanford.edu/business-podcasts/all-else-equal-making-better-decisions)
+Stanford GSB Quick Study Videos – finance research (gsb.stanford.edu/business-videos/quick-study)
+★ GENERAL:
+Aswath Damodaran – Valuation MBA Spring 2025 (YT: youtube.com/playlist?list=PLUkh9m2BorqkgpNyRpP-NL3BS4yvFabXk)
 Patrick Boyle – On Finance (YT: youtube.com/@PBoyle)
 Corporate Finance Institute – CFI (YT: youtube.com/channel/UCGtbVv_ACgV7difdVZ92NMw)</t>
         </is>
       </c>
       <c r="L11" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
+          <t>★ STANFORD OFFICIAL:
+Stanford Online MS&amp;E 276 Entrepreneurial Management &amp; Finance (online.stanford.edu/courses/mse276-entrepreneurial-management-and-finance)
+Stanford LEAD Program ~$19,200 – covers financial valuation module (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
 Wharton Finance on Coursera – free audit / $49 cert (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
@@ -1463,7 +1487,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="66" t="n"/>
+      <c r="A13" s="7" t="n"/>
       <c r="B13" s="71" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -1523,7 +1547,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="66" t="n"/>
+      <c r="A14" s="7" t="n"/>
       <c r="B14" s="71" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1571,18 +1595,27 @@
       </c>
       <c r="K14" s="65" t="inlineStr">
         <is>
-          <t>Marginal Revolution University – Principles of Microeconomics (mru.org/courses/principles-of-microeconomics)
+          <t>★ STANFORD OFFICIAL:
+Stanford Coursera Game Theory – Matthew Jackson (free audit; coursera.org/learn/game-theory-1)
+Stanford Game Theory II – Advanced (free audit; coursera.org/learn/game-theory-2)
+Stanford edX Principles of Economics (free audit; edx.org/learn/economics/stanford-university-principles-of-economics)
+If/Then Podcast – economics &amp; pricing research episodes (gsb.stanford.edu/business-podcasts/if-then)
+★ GENERAL:
+Marginal Revolution University – Principles of Microeconomics (mru.org/courses/principles-of-microeconomics)
 Khan Academy Microeconomics (khanacademy.org/economics-finance-domain/microeconomics)</t>
         </is>
       </c>
       <c r="L14" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 – economics &amp; decision-making module (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="66" t="n"/>
+      <c r="A15" s="7" t="n"/>
       <c r="B15" s="71" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1630,19 +1663,26 @@
       </c>
       <c r="K15" s="65" t="inlineStr">
         <is>
-          <t>Marginal Revolution University – Principles of Macroeconomics (mru.org/courses/principles-of-macroeconomics)
+          <t>★ STANFORD OFFICIAL:
+Stanford edX Principles of Economics – covers macro (free audit; edx.org/learn/economics/stanford-university-principles-of-economics)
+If/Then Podcast – macro &amp; policy research episodes (gsb.stanford.edu/business-podcasts/if-then)
+★ GENERAL:
+Marginal Revolution University – Principles of Macroeconomics (mru.org/courses/principles-of-macroeconomics)
 Economics Explained (YT: youtube.com/c/EconomicsExplained)
 Khan Academy Macroeconomics (khanacademy.org/economics-finance-domain/macroeconomics)</t>
         </is>
       </c>
       <c r="L15" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="67" t="n"/>
+      <c r="A16" s="8" t="n"/>
       <c r="B16" s="71" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1690,14 +1730,24 @@
       </c>
       <c r="K16" s="65" t="inlineStr">
         <is>
-          <t>Freakonomics Radio – business &amp; political economy episodes (freakonomics.com)
+          <t>★ STANFORD OFFICIAL:
+POLECON 239 Syllabus 2017 PDF – Saumitra Jha (web.stanford.edu/~saumitra/docs/POLECON239syllabus2017_1.pdf)
+Anat Admati – Finance &amp; Society Syllabus PDF (gsb-faculty.stanford.edu/anat-r-admati)
+Stanford GSB View From The Top – policy &amp; leadership talks [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+Stanford Social Innovation Review (ssir.org)
+Stanford eCorner – regulation &amp; innovation talks (ecorner.stanford.edu)
+★ GENERAL:
+Freakonomics Radio – business &amp; political economy episodes (freakonomics.com)
 HBS Cold Call Podcast – ethics &amp; policy cases (hbr.org/2019/04/podcast-cold-call)
 HBR IdeaCast Podcast (hbr.org/podcasts)</t>
         </is>
       </c>
       <c r="L16" s="65" t="inlineStr">
         <is>
-          <t>— (no direct HBS Online equivalent)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford Executive Program in Strategy &amp; Organization (gsb.stanford.edu/exec-ed/programs/executive-program-strategy-organization)
+★ OTHER PAID:
+— (no direct HBS Online equivalent)</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1813,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="66" t="n"/>
+      <c r="A18" s="7" t="n"/>
       <c r="B18" s="73" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -1823,7 +1873,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="67" t="n"/>
+      <c r="A19" s="8" t="n"/>
       <c r="B19" s="73" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -1867,13 +1917,21 @@
       <c r="J19" s="73" t="inlineStr"/>
       <c r="K19" s="65" t="inlineStr">
         <is>
-          <t>HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Class Takeaways – Marketing &amp; consumer behavior episodes [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+If/Then Podcast – marketing research episodes (gsb.stanford.edu/business-podcasts/if-then)
+Stanford eCorner – go-to-market &amp; growth talks (ecorner.stanford.edu)
+★ GENERAL:
+HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
 Neil Patel – Digital Marketing Strategy (YT: youtube.com/neilpatel)</t>
         </is>
       </c>
       <c r="L19" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 – includes marketing module (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)
 Wharton Marketing on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
@@ -1939,7 +1997,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="66" t="n"/>
+      <c r="A21" s="7" t="n"/>
       <c r="B21" s="75" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -1999,7 +2057,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="67" t="n"/>
+      <c r="A22" s="8" t="n"/>
       <c r="B22" s="75" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2043,13 +2101,20 @@
       <c r="J22" s="75" t="inlineStr"/>
       <c r="K22" s="65" t="inlineStr">
         <is>
-          <t>MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
+          <t>★ STANFORD OFFICIAL:
+MS&amp;E 348 Course Page – related optimization content (web.stanford.edu/class/msande348/)
+Stanford GSB Quick Study Videos – operations research (gsb.stanford.edu/business-videos/quick-study)
+★ GENERAL:
+MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
 Wharton Operations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
       <c r="L22" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2184,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="66" t="n"/>
+      <c r="A24" s="7" t="n"/>
       <c r="B24" s="77" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -2176,7 +2241,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="66" t="n"/>
+      <c r="A25" s="7" t="n"/>
       <c r="B25" s="77" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2224,19 +2289,27 @@
       </c>
       <c r="K25" s="65" t="inlineStr">
         <is>
-          <t>StatQuest with Josh Starmer (YT: youtube.com/c/joshstarmer)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Class Takeaways – Data-Driven Decision Making (Prof. Mohsen Bayati) [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+All Else Equal Podcast – decision-making &amp; analytics (gsb.stanford.edu/business-podcasts/all-else-equal-making-better-decisions)
+★ GENERAL:
+StatQuest with Josh Starmer (YT: youtube.com/c/joshstarmer)
 Alex The Analyst (YT: youtube.com/@AlexTheAnalyst)
 Khan Academy Statistics (khanacademy.org/math/statistics-probability)</t>
         </is>
       </c>
       <c r="L25" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB ExecEd Data-Driven Decision Making (gsb.stanford.edu/exec-ed/programs/data-driven-decision-making)
+Stanford GSB Demystify Decision Making (gsb.stanford.edu/exec-ed/programs/demystify-decision-making)
+★ OTHER PAID:
+HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="66" t="n"/>
+      <c r="A26" s="7" t="n"/>
       <c r="B26" s="77" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2280,18 +2353,25 @@
       <c r="J26" s="77" t="inlineStr"/>
       <c r="K26" s="65" t="inlineStr">
         <is>
-          <t>StatQuest with Josh Starmer – ML/optimization concepts (YT: youtube.com/c/joshstarmer)
+          <t>★ STANFORD OFFICIAL:
+MS&amp;E 348 Course Page – decision trees, stochastic programming, Monte Carlo (web.stanford.edu/class/msande348/)
+Stanford edX – quantitative methods content (edx.org/school/stanfordonline)
+★ GENERAL:
+StatQuest with Josh Starmer – ML/optimization concepts (YT: youtube.com/c/joshstarmer)
 365 Data Science (YT: youtube.com/c/365DataScience)</t>
         </is>
       </c>
       <c r="L26" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Demystify Decision Making (gsb.stanford.edu/exec-ed/programs/demystify-decision-making)
+★ OTHER PAID:
+HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="67" t="n"/>
+      <c r="A27" s="8" t="n"/>
       <c r="B27" s="77" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2335,13 +2415,21 @@
       <c r="J27" s="77" t="inlineStr"/>
       <c r="K27" s="65" t="inlineStr">
         <is>
-          <t>HBR IdeaCast – Digital transformation episodes (hbr.org/podcasts)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB View From The Top – technology leadership talks [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+If/Then Podcast – AI &amp; technology research (gsb.stanford.edu/business-podcasts/if-then)
+Stanford eCorner – digital transformation &amp; platform talks (ecorner.stanford.edu)
+★ GENERAL:
+HBR IdeaCast – Digital transformation episodes (hbr.org/podcasts)
 Stanford GSB YouTube – technology strategy talks (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
         </is>
       </c>
       <c r="L27" s="65" t="inlineStr">
         <is>
-          <t>— (no direct HBS Online equivalent)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford Online MS&amp;E 280 Organizational Behavior (includes IT strategy module; online.stanford.edu/courses/mse280-organizational-behavior-evidence-action)
+★ OTHER PAID:
+— (no direct HBS Online equivalent)</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2496,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="66" t="n"/>
+      <c r="A29" s="7" t="n"/>
       <c r="B29" s="79" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -2469,7 +2557,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="67" t="n"/>
+      <c r="A30" s="8" t="n"/>
       <c r="B30" s="79" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2513,14 +2601,25 @@
       <c r="J30" s="79" t="inlineStr"/>
       <c r="K30" s="65" t="inlineStr">
         <is>
-          <t>Modern MBA (YT: youtube.com/c/ModernMBA)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB View From The Top [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+Think Fast Talk Smart Podcast – 200+ episodes on leadership &amp; communication (gsb.stanford.edu/business-podcasts/think-fast-talk-smart-podcast / fastersmarter.io)
+Jeffrey Pfeffer OB 377 Course Outline 2024 PDF (jeffreypfeffer.com/wp-content/uploads/2024/08/CourseOutline2024.pdf)
+Stanford eCorner – leadership &amp; scaling talks (ecorner.stanford.edu)
+★ GENERAL:
+Modern MBA (YT: youtube.com/c/ModernMBA)
 Stanford GSB YouTube – strategy talks (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)
 HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)</t>
         </is>
       </c>
       <c r="L30" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 – core strategic leadership focus (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+Stanford Online Discover Paths to Power ~$1,500 – Jeffrey Pfeffer (online.stanford.edu/courses/gsb-x0013-discover-paths-power)
+Stanford Executive Program in Strategy &amp; Organization (gsb.stanford.edu/exec-ed/programs/executive-program-strategy-organization)
+★ OTHER PAID:
+HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2687,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="66" t="n"/>
+      <c r="A32" s="7" t="n"/>
       <c r="B32" s="81" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -2645,7 +2744,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="66" t="n"/>
+      <c r="A33" s="7" t="n"/>
       <c r="B33" s="81" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2689,7 +2788,13 @@
       <c r="J33" s="81" t="inlineStr"/>
       <c r="K33" s="65" t="inlineStr">
         <is>
-          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+          <t>★ STANFORD OFFICIAL:
+Coursera Organizational Analysis – Stanford (free audit, 4.6★, 78k+ enrolled; coursera.org/learn/organizational-analysis)
+Stanford GSB View From The Top [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+Stanford GSB Class Takeaways – Team Management &amp; Humor in Business [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+Think Fast Talk Smart Podcast (gsb.stanford.edu/business-podcasts/think-fast-talk-smart-podcast)
+★ GENERAL:
+Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
 HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)
 Stanford GSB YouTube (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)
 TED Business (YT: youtube.com/c/TEDBusiness)</t>
@@ -2697,12 +2802,18 @@
       </c>
       <c r="L33" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford Online MS&amp;E 280 Organizational Behavior – Evidence in Action (Stanford credit; online.stanford.edu/courses/mse280-organizational-behavior-evidence-action)
+Stanford GSB Managing Teams for Innovation &amp; Success (gsb.stanford.edu/exec-ed/programs/managing-teams-innovation-success)
+Stanford Online Discover Paths to Power ~$1,500 (online.stanford.edu/courses/gsb-x0013-discover-paths-power)
+Stanford Online Influence &amp; Negotiation Strategies (online.stanford.edu/courses/gsb-x0007-influence-and-negotiation-strategies-program)
+★ OTHER PAID:
+HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="67" t="n"/>
+      <c r="A34" s="8" t="n"/>
       <c r="B34" s="81" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2746,13 +2857,21 @@
       <c r="J34" s="81" t="inlineStr"/>
       <c r="K34" s="65" t="inlineStr">
         <is>
-          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Class Takeaways – Talent &amp; Culture episodes [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+If/Then Podcast – future of work &amp; talent research (gsb.stanford.edu/business-podcasts/if-then)
+Stanford GSB Quick Study Videos – HR research (gsb.stanford.edu/business-videos/quick-study)
+★ GENERAL:
+Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
 HBR IdeaCast Podcast – people &amp; talent episodes (hbr.org/podcasts)</t>
         </is>
       </c>
       <c r="L34" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB Managing Teams for Innovation &amp; Success (gsb.stanford.edu/exec-ed/programs/managing-teams-innovation-success)
+★ OTHER PAID:
+HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2937,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="66" t="n"/>
+      <c r="A36" s="7" t="n"/>
       <c r="B36" s="83" t="inlineStr">
         <is>
           <t>HBS</t>
@@ -2878,7 +2997,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="67" t="n"/>
+      <c r="A37" s="8" t="n"/>
       <c r="B37" s="83" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -2922,14 +3041,22 @@
       <c r="J37" s="83" t="inlineStr"/>
       <c r="K37" s="65" t="inlineStr">
         <is>
-          <t>HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)
+          <t>★ STANFORD OFFICIAL:
+Stanford GSB View From The Top – values &amp; ethics episodes [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+Stanford GSB Class Takeaways – Leading with Values (Profs. Malhotra &amp; Shotts) [YT: youtube.com/playlist?list=PLxq_lXOUlvQCrEwiwPaUSJoUzIDTUnq2_]
+Stanford Social Innovation Review (ssir.org)
+★ GENERAL:
+HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)
 TED Business (YT: youtube.com/c/TEDBusiness)
 HBR IdeaCast Podcast (hbr.org/podcasts)</t>
         </is>
       </c>
       <c r="L37" s="65" t="inlineStr">
         <is>
-          <t>— (no direct HBS Online equivalent)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 – includes ethics &amp; values module (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+— (no direct HBS Online equivalent)</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3250,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="66" t="n"/>
+      <c r="A41" s="7" t="n"/>
       <c r="B41" s="89" t="inlineStr">
         <is>
           <t>HBS</t>
@@ -3181,7 +3308,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="66" t="n"/>
+      <c r="A42" s="7" t="n"/>
       <c r="B42" s="89" t="inlineStr">
         <is>
           <t>MIT Sloan</t>
@@ -3239,7 +3366,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="66" t="n"/>
+      <c r="A43" s="7" t="n"/>
       <c r="B43" s="89" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -3287,18 +3414,25 @@
       </c>
       <c r="K43" s="65" t="inlineStr">
         <is>
-          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+          <t>★ STANFORD OFFICIAL:
+Think Fast Talk Smart Podcast – 200+ communication &amp; leadership episodes (gsb.stanford.edu/business-podcasts/think-fast-talk-smart-podcast / fastersmarter.io)
+Stanford GSB View From The Top [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+★ GENERAL:
+Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
 Stanford GSB YouTube (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
         </is>
       </c>
       <c r="L43" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford Online Influence &amp; Negotiation Strategies (online.stanford.edu/courses/gsb-x0007-influence-and-negotiation-strategies-program)
+★ OTHER PAID:
+HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="67" t="n"/>
+      <c r="A44" s="8" t="n"/>
       <c r="B44" s="89" t="inlineStr">
         <is>
           <t>Stanford GSB</t>
@@ -3346,12 +3480,20 @@
       </c>
       <c r="K44" s="65" t="inlineStr">
         <is>
-          <t>— (global immersion requirement; no direct online equivalent)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford eCorner – global entrepreneurship &amp; emerging markets talks (ecorner.stanford.edu)
+Stanford Social Innovation Review – global development (ssir.org)
+Stanford GSB View From The Top – global leaders [YT: youtube.com/playlist?list=PLxq_lXOUlvQAwaY_9K4ZFH9Xdar9WzCaL]
+★ GENERAL:
+— (global immersion requirement; no direct online equivalent)</t>
         </is>
       </c>
       <c r="L44" s="65" t="inlineStr">
         <is>
-          <t>— (global immersion requirement; no direct online equivalent)</t>
+          <t>★ STANFORD OFFICIAL:
+Stanford LEAD Program ~$19,200 – global cohort &amp; virtual immersion (gsb.stanford.edu/exec-ed/programs/stanford-lead)
+★ OTHER PAID:
+— (global immersion requirement; no direct online equivalent)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add MIT Sloan-specific official resources to all 10 MIT course rows
Prepended MIT-official resources (★ MIT OFFICIAL section) to Free and Paid
columns for all 10 MIT Sloan first-year courses, covering: MIT OCW courses
with full materials (15.401 with video lectures, 15.501, 15.010, 15.060,
15.761, 15.311, 15.280), MIT Sloan 15.900 syllabus PDF, OCW substitutes for
courses not on OCW (15.902, 15.963 for strategy; 15.810 for marketing),
MITx/edX paid and free-audit courses (MicroMasters in Finance, Financial
Accounting, Foundations of Modern Finance), MIT ExecEd programs, MIT Sloan
Management Review, Ideas Made to Matter series, and Data Made to Matter podcast.

https://claude.ai/code/session_011QHxcNSM1P2957ocCew2SU
</commit_message>
<xml_diff>
--- a/m7_year1_master_by_topic.xlsx
+++ b/m7_year1_master_by_topic.xlsx
@@ -1035,14 +1035,24 @@
       <c r="J5" s="64" t="inlineStr"/>
       <c r="K5" s="65" t="inlineStr">
         <is>
-          <t>Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
+          <t>★ MIT OFFICIAL (OCW – FREE):
+MIT OCW 15.501 Intro to Financial &amp; Managerial Accounting – lecture notes, 7 problem sets + solutions, 3 exams + solutions (ocw.mit.edu/courses/15-501-introduction-to-financial-and-managerial-accounting-spring-2004/)
+MIT OCW 15.515 Financial Accounting – lecture notes, assignments (ocw.mit.edu/courses/15-515-financial-accounting-fall-2003/)
+MIT OCW Collection – MBA First-Semester Core (ocw.mit.edu/collections/sloan-mba-first-semester-core/)
+MIT Ideas Made to Matter – accounting &amp; finance articles (mitsloan.mit.edu/ideas-made-to-matter)
+★ GENERAL:
+Edspira (YT: youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg)
 MIT OCW Financial Accounting 15.515 (ocw.mit.edu/courses/15-515-financial-accounting-fall-2003/)
 Khan Academy Finance &amp; Accounting (khanacademy.org/economics-finance-domain/core-finance)</t>
         </is>
       </c>
       <c r="L5" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
+          <t>★ MIT OFFICIAL (PAID):
+MITx Financial Accounting on edX – free audit / ~$300 cert (edx.org/learn/financial-accounting/massachusetts-institute-of-technology-financial-accounting)
+MITx MicroMasters in Finance – includes Financial Accounting (edx.org/micromasters/mitx-finance)
+★ OTHER PAID:
+HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
@@ -1343,14 +1353,27 @@
       </c>
       <c r="K10" s="65" t="inlineStr">
         <is>
-          <t>Aswath Damodaran – Corporate Finance Full Course (YT: youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw)
+          <t>★ MIT OFFICIAL (OCW – FREE) — Crown Jewel:
+MIT OCW 15.401 Finance Theory I – FULL VIDEO LECTURES (all 12 modules, 90 min each), slides, recitation notes, problem sets + solutions, exams (ocw.mit.edu/courses/15-401-finance-theory-i-fall-2008/)
+YouTube Playlist – 15.401 Full Lectures by Prof. Andrew Lo (youtube.com/playlist?list=PLUl4u3cNGP63B2lDhyKOsImI7FjCf6eDW)
+Internet Archive backup: archive.org/details/MIT15.401F08
+Prof. Andrew Lo Teaching Page + 2018 syllabus (alo.mit.edu/teaching/)
+MIT OCW 15.481x Adaptive Markets – videos, problem sets (ocw.mit.edu/courses/15-481x-adaptive-markets-financial-market-dynamics-and-human-behavior-fall-2022/)
+★ GENERAL:
+Aswath Damodaran – Corporate Finance Full Course (YT: youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw)
 Patrick Boyle – On Finance (YT: youtube.com/@PBoyle)
 Corporate Finance Institute – CFI (YT: youtube.com/channel/UCGtbVv_ACgV7difdVZ92NMw)</t>
         </is>
       </c>
       <c r="L10" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
+          <t>★ MIT OFFICIAL (PAID):
+MITx Foundations of Modern Finance I – free audit / ~$300 cert (edx.org/learn/finance/massachusetts-institute-of-technology-foundations-of-modern-finance-i)
+MITx Foundations of Modern Finance II (edx.org/learn/finance/massachusetts-institute-of-technology-foundations-of-modern-finance-ii)
+MITx MicroMasters in Finance – 5-course program, graduate-level (edx.org/micromasters/mitx-finance)
+MIT ExecEd Fundamentals of Finance for Technical Executives (executive.mit.edu/course/fundamentals-of-finance-for-the-technical-executive/a056g00000URaMtAAL.html)
+★ OTHER PAID:
+HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)
 Wharton Finance on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
@@ -1535,14 +1558,22 @@
       </c>
       <c r="K13" s="65" t="inlineStr">
         <is>
-          <t>Marginal Revolution University – Microeconomics (mru.org)
+          <t>★ MIT OFFICIAL (OCW – FREE):
+MIT OCW 15.010 Economic Analysis for Business Decisions – full lecture notes, 6 homework sets + solutions, 6 years of final exams + solutions (ocw.mit.edu/courses/15-010-economic-analysis-for-business-decisions-fall-2004/)
+Covers: market definition, pricing strategy, oligopoly, game theory, auctions, antitrust, asymmetric information
+Textbook: Pindyck &amp; Rubinfeld Microeconomics (publicly referenced)
+★ GENERAL:
+Marginal Revolution University – Microeconomics (mru.org)
 Khan Academy Microeconomics (khanacademy.org/economics-finance-domain/microeconomics)
 Freakonomics Radio Podcast (freakonomics.com)</t>
         </is>
       </c>
       <c r="L13" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd Systems Thinking &amp; Complex Problem Solving (executive.mit.edu/course/understanding-and-solving-complex-business-problems/a046g00000PI9BcAAL.html)
+★ OTHER PAID:
+HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
     </row>
@@ -1861,14 +1892,24 @@
       </c>
       <c r="K18" s="65" t="inlineStr">
         <is>
-          <t>HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
+          <t>★ MIT OFFICIAL (FREE):
+Prof. John Hauser Faculty Page – 15.814 assignments, problem sets, pricing &amp; promotions exercises, 2018 syllabus PDF (mitmgmtfaculty.mit.edu/jhauser/course_materials/)
+Direct syllabus PDF: mit.edu/~hauser/Pages/Syllabus%2015.814%20Fall%202018%20May%2021.pdf
+MIT OCW 15.810 Marketing Management Fall 2015 – lecture notes, readings (ocw.mit.edu/courses/15-810-marketing-management-analytics-frameworks-and-applications-fall-2015/)
+MIT OCW 15.810 Marketing Management Fall 2010 – lecture notes, projects (ocw.mit.edu/courses/15-810-marketing-management-fall-2010/)
+MIT Ideas Made to Matter – marketing &amp; consumer behavior articles (mitsloan.mit.edu/ideas-made-to-matter)
+★ GENERAL:
+HubSpot Marketing YouTube + HubSpot Academy (youtube.com/user/HubSpot; academy.hubspot.com)
 Neil Patel – Digital Marketing Strategy (YT: youtube.com/neilpatel)
 Wharton Marketing on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
       <c r="L18" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)</t>
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd – Marketing &amp; Strategy programs (executive.mit.edu)
+★ OTHER PAID:
+HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)</t>
         </is>
       </c>
     </row>
@@ -2045,13 +2086,22 @@
       </c>
       <c r="K21" s="65" t="inlineStr">
         <is>
-          <t>MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
+          <t>★ MIT OFFICIAL (OCW – FREE):
+MIT OCW 15.761 Intro to Operations Management Spring 2013 – cases, simulation exercises, assignments (ocw.mit.edu/courses/15-761-introduction-to-operations-management-spring-2013/)
+MIT OCW 15.760b Intro to Operations Management Spring 2004 – full lecture notes PDFs (~19 lectures: process flow, Little's Law, inventory, queuing, supply chains) (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
+Textbook: Cachon &amp; Terwiesch Matching Supply with Demand (referenced)
+MIT Ideas Made to Matter – operations &amp; supply chain articles (mitsloan.mit.edu/ideas-made-to-matter)
+★ GENERAL:
+MIT OCW Intro to Operations Management 15.760B (ocw.mit.edu/courses/15-760b-introduction-to-operations-management-spring-2004/)
 Wharton Operations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
       <c r="L21" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd System Dynamics &amp; Business Dynamics (executive.mit.edu/course/business-dynamics/a056g00000URaMkAAL.html)
+★ OTHER PAID:
+HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)
 Wharton Operations on Coursera ~$49 cert</t>
         </is>
       </c>
@@ -2228,14 +2278,26 @@
       <c r="J24" s="77" t="inlineStr"/>
       <c r="K24" s="65" t="inlineStr">
         <is>
-          <t>StatQuest with Josh Starmer – Statistics &amp; ML (YT: youtube.com/c/joshstarmer)
+          <t>★ MIT OFFICIAL (OCW – FREE):
+MIT OCW 15.060 Data, Models &amp; Decisions Fall 2014 – syllabus, lecture summaries, 7 homework sets + solutions (probability, simulation, regression, linear optimization, discrete optimization) (ocw.mit.edu/courses/15-060-data-models-and-decisions-fall-2014/)
+MIT OCW 15.071 The Analytics Edge Spring 2017 – WITH VIDEO LECTURES; covers regression, trees, text analytics, optimization, visualization (ocw.mit.edu/courses/15-071-the-analytics-edge-spring-2017/)
+MIT OCW 15.063 Communicating With Data Summer 2003 (ocw.mit.edu/courses/15-063-communicating-with-data-summer-2003/)
+MIT Open Learning Library 15.481x Adaptive Markets – free interactive (openlearninglibrary.mit.edu/courses/course-v1:MITx+15.481x+1T2021/about)
+MIT Ideas Made to Matter – data &amp; AI articles (mitsloan.mit.edu/ideas-made-to-matter)
+Data Made to Matter Podcast (mitsloan.mit.edu/podcast)
+★ GENERAL:
+StatQuest with Josh Starmer – Statistics &amp; ML (YT: youtube.com/c/joshstarmer)
 Alex The Analyst (YT: youtube.com/@AlexTheAnalyst)
 Khan Academy Statistics &amp; Probability (khanacademy.org/math/statistics-probability)</t>
         </is>
       </c>
       <c r="L24" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)
+          <t>★ MIT OFFICIAL (PAID):
+MITx Mathematical Methods for Quantitative Finance – free audit (edx.org/micromasters/mitx-finance)
+MIT ExecEd Systems Thinking Courses (executive.mit.edu/systems-thinking)
+★ OTHER PAID:
+HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)
 HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
         </is>
       </c>
@@ -2544,14 +2606,24 @@
       </c>
       <c r="K29" s="65" t="inlineStr">
         <is>
-          <t>Modern MBA (YT: youtube.com/c/ModernMBA)
+          <t>★ MIT OFFICIAL (FREE):
+MIT Sloan 15.900 Official Syllabus PDF Fall 2022 – full session list, case list (Apple, Southwest, Zara, Netflix, Disney, Danaher) (mitsloan.mit.edu/sites/default/files/inline-files/Comp%20Strat%202022%20syllabus%2010%20AUG%2022%5B46%5D.pdf)
+MIT OCW 15.902 Strategic Management I – full lecture notes (Delta Model, Porter, RBV, competitive positioning) (ocw.mit.edu/courses/15-902-strategic-management-i-fall-2006/)
+MIT OCW 15.963 Advanced Strategy – lecture notes incl. '15.900 Review: Strategy Fundamentals' (ocw.mit.edu/courses/15-963-advanced-strategy-spring-2008/)
+MIT Sloan Management Review – strategy articles (sloanreview.mit.edu)
+MIT Ideas Made to Matter – strategy research (mitsloan.mit.edu/ideas-made-to-matter)
+★ GENERAL:
+Modern MBA (YT: youtube.com/c/ModernMBA)
 Acquired Podcast (acquired.fm)
 HBS Cold Call Podcast (hbr.org/2019/04/podcast-cold-call)</t>
         </is>
       </c>
       <c r="L29" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd Executive Program in Strategy &amp; Organization (executive.mit.edu)
+★ OTHER PAID:
+HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)
 Wharton Business Foundations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
@@ -2731,14 +2803,26 @@
       <c r="J32" s="81" t="inlineStr"/>
       <c r="K32" s="65" t="inlineStr">
         <is>
-          <t>Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
+          <t>★ MIT OFFICIAL (OCW – FREE):
+MIT OCW 15.311 Organizational Processes Fall 2003 – syllabus, readings list (org power, networks, culture, strategy design), assignments, team project description (ocw.mit.edu/courses/15-311-organizational-processes-fall-2003/)
+MIT OCW 15.317 Organizational Leadership &amp; Change Summer 2009 (ocw.mit.edu/courses/15-317-organizational-leadership-and-change-summer-2009/)
+Prof. John Sterman – Business Dynamics page &amp; textbook info (mitmgmtfaculty.mit.edu/jsterman/)
+MIT Sloan Management Review – org behavior &amp; leadership articles (sloanreview.mit.edu)
+Data Made to Matter Podcast (mitsloan.mit.edu/podcast)
+MITx Shaping Work of the Future – free audit on edX (edx.org/learn/human-resources/massachusetts-institute-of-technology-shaping-work-of-the-future)
+★ GENERAL:
+Simon Sinek YouTube (youtube.com/channel/UCBKbem_ewc4TVHBzE2Jp9Hg)
 HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)
 HBR IdeaCast Podcast (hbr.org/podcasts)</t>
         </is>
       </c>
       <c r="L32" s="65" t="inlineStr">
         <is>
-          <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd System Dynamics &amp; Business Dynamics (executive.mit.edu/course/business-dynamics/a056g00000URaMkAAL.html)
+MIT ExecEd Organizations &amp; Leadership courses (executive.mit.edu/organizations-and-leadership)
+★ OTHER PAID:
+HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)
 HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
         </is>
       </c>
@@ -3177,13 +3261,21 @@
       </c>
       <c r="K39" s="65" t="inlineStr">
         <is>
-          <t>TED Business – communication &amp; presentation talks (YT: youtube.com/c/TEDBusiness)
+          <t>★ MIT OFFICIAL (OCW – FREE):
+MIT OCW 15.280 Communication for Managers Fall 2016 – syllabus, readings, team presentation project, strategic communicator reflection assignment (ocw.mit.edu/courses/15-280-communication-for-managers-fall-2016/)
+MIT OCW 15.281 Advanced Communication for Leaders Spring 2016 (ocw.mit.edu/courses/sloan-school-of-management/15-281-advanced-communication-for-leaders-spring-2016/)
+MIT Ideas Made to Matter – communication &amp; leadership articles (mitsloan.mit.edu/ideas-made-to-matter)
+★ GENERAL:
+TED Business – communication &amp; presentation talks (YT: youtube.com/c/TEDBusiness)
 Stanford GSB YouTube – communication &amp; public speaking (youtube.com/channel/UCGwuxdEeCf0TIA2RbPOj-8g)</t>
         </is>
       </c>
       <c r="L39" s="65" t="inlineStr">
         <is>
-          <t>— (no direct HBS Online equivalent)</t>
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd Organizations &amp; Leadership courses (executive.mit.edu/organizations-and-leadership)
+★ OTHER PAID:
+— (no direct HBS Online equivalent)</t>
         </is>
       </c>
     </row>
@@ -3356,12 +3448,22 @@
       </c>
       <c r="K42" s="65" t="inlineStr">
         <is>
-          <t>HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)</t>
+          <t>★ MIT OFFICIAL (FREE – closest proxies; 15.002 itself has no public materials):
+MIT OCW 15.317 Organizational Leadership &amp; Change Summer 2009 (ocw.mit.edu/courses/15-317-organizational-leadership-and-change-summer-2009/)
+MIT OCW 15.974 Practical Leadership Fall 2004 (ocw.mit.edu/courses/sloan-school-of-management/15-974-practical-leadership-fall-2004/)
+MIT Sloan Management Review – inclusion &amp; leadership articles (sloanreview.mit.edu)
+MITx Shaping Work of the Future – free audit on edX (edx.org/learn/human-resources/massachusetts-institute-of-technology-shaping-work-of-the-future)
+Sloanies Talking with Sloanies Podcast (mitsloan.mit.edu/alumni/sloanies-talking-sloanies)
+★ GENERAL:
+HarvardX Exercising Leadership – free audit on edX (edx.org/learn/leadership/harvard-university-exercising-leadership-foundational-principles)</t>
         </is>
       </c>
       <c r="L42" s="65" t="inlineStr">
         <is>
-          <t>— (immersive off-campus; no direct online equivalent)</t>
+          <t>★ MIT OFFICIAL (PAID):
+MIT ExecEd Organizations &amp; Leadership courses (executive.mit.edu/organizations-and-leadership)
+★ OTHER PAID:
+— (immersive off-campus; no direct online equivalent)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Recommended Starter Course column (M) to all 41 course rows
Added a 13th column — 'Recommended Starter Course (Try This First)' — across
all 12 topic groups. Each recommendation is the single best free (or lowest-
cost) resource to test interest in that field before committing to a career,
with rationale and career outcomes. Covers: Edspira (Accounting), Damodaran
(Finance), MRU (Economics), HubSpot Academy (Marketing), MIT OCW 15.761
(Operations), Alex The Analyst (Data/AI), Modern MBA (Strategy), Stanford
Coursera Org Analysis (Leadership/OB), Sandel Justice (Ethics), YC Startup
School (Entrepreneurship), Stanford Think Fast Talk Smart (Communication),
Stanford eCorner (Experiential/Global).

https://claude.ai/code/session_011QHxcNSM1P2957ocCew2SU
</commit_message>
<xml_diff>
--- a/m7_year1_master_by_topic.xlsx
+++ b/m7_year1_master_by_topic.xlsx
@@ -65,7 +65,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -147,6 +147,11 @@
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -207,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -468,6 +473,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -835,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -850,6 +858,7 @@
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -927,6 +936,11 @@
           <t>Paid Resources (HBS Online / Coursera)</t>
         </is>
       </c>
+      <c r="M3" s="90" t="inlineStr">
+        <is>
+          <t>⭐ Recommended Starter Course (Try This First)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
@@ -987,6 +1001,16 @@
         <is>
           <t>HBS Online Financial Accounting ~$1,750 (online.hbs.edu/courses/financial-accounting)
 HBS Online CORe Bundle ~$2,650 – includes Financial Accounting (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
+      <c r="M4" s="65" t="inlineStr">
+        <is>
+          <t>Edspira – Financial Accounting Playlist
+FREE · YouTube
+youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg
+Why: Prof. McLaughlin (PhD, CPA) makes the 'language of business' click in
+10-min bites. Sample 8–10 videos — accounting either grabs you or it doesn't.
+🎯 Careers if it clicks: CFO track, FP&amp;A, audit, financial analyst, controller.</t>
         </is>
       </c>
     </row>
@@ -1056,6 +1080,16 @@
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M5" s="65" t="inlineStr">
+        <is>
+          <t>Edspira – Financial Accounting Playlist
+FREE · YouTube
+youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg
+Why: Prof. McLaughlin (PhD, CPA) makes the 'language of business' click in
+10-min bites. Sample 8–10 videos — accounting either grabs you or it doesn't.
+🎯 Careers if it clicks: CFO track, FP&amp;A, audit, financial analyst, controller.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -1121,6 +1155,16 @@
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M6" s="65" t="inlineStr">
+        <is>
+          <t>Edspira – Financial Accounting Playlist
+FREE · YouTube
+youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg
+Why: Prof. McLaughlin (PhD, CPA) makes the 'language of business' click in
+10-min bites. Sample 8–10 videos — accounting either grabs you or it doesn't.
+🎯 Careers if it clicks: CFO track, FP&amp;A, audit, financial analyst, controller.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>
@@ -1185,6 +1229,16 @@
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M7" s="65" t="inlineStr">
+        <is>
+          <t>Edspira – Financial Accounting Playlist
+FREE · YouTube
+youtube.com/channel/UCzRF-OFuv8os-bGzANpQGqg
+Why: Prof. McLaughlin (PhD, CPA) makes the 'language of business' click in
+10-min bites. Sample 8–10 videos — accounting either grabs you or it doesn't.
+🎯 Careers if it clicks: CFO track, FP&amp;A, audit, financial analyst, controller.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="68" t="inlineStr">
@@ -1247,6 +1301,18 @@
 HBS Online CORe Bundle ~$2,650 (online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M8" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Corporate Finance Full Course ⭐
+FREE · YouTube
+youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw
+Why: The 'Dean of Valuation' posts his entire NYU Stern MBA semester online.
+Highest-signal test — if the first 5 sessions energize you, finance is your field.
+Nothing freely available comes close in rigor or completeness.
+🎯 Careers if it clicks: Investment banking, PE/VC, equity research, asset
+management, corporate development, M&amp;A.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1301,6 +1367,18 @@
       <c r="L9" s="65" t="inlineStr">
         <is>
           <t>HBS Online Leading with Finance ~$1,750 (online.hbs.edu/courses/leading-with-finance)</t>
+        </is>
+      </c>
+      <c r="M9" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Corporate Finance Full Course ⭐
+FREE · YouTube
+youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw
+Why: The 'Dean of Valuation' posts his entire NYU Stern MBA semester online.
+Highest-signal test — if the first 5 sessions energize you, finance is your field.
+Nothing freely available comes close in rigor or completeness.
+🎯 Careers if it clicks: Investment banking, PE/VC, equity research, asset
+management, corporate development, M&amp;A.</t>
         </is>
       </c>
     </row>
@@ -1377,6 +1455,18 @@
 Wharton Finance on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
+      <c r="M10" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Corporate Finance Full Course ⭐
+FREE · YouTube
+youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw
+Why: The 'Dean of Valuation' posts his entire NYU Stern MBA semester online.
+Highest-signal test — if the first 5 sessions energize you, finance is your field.
+Nothing freely available comes close in rigor or completeness.
+🎯 Careers if it clicks: Investment banking, PE/VC, equity research, asset
+management, corporate development, M&amp;A.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
@@ -1443,6 +1533,18 @@
 Wharton Finance on Coursera – free audit / $49 cert (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
+      <c r="M11" s="65" t="inlineStr">
+        <is>
+          <t>Aswath Damodaran – Corporate Finance Full Course ⭐
+FREE · YouTube
+youtube.com/channel/UCLvnJL8htRR1T9cbSccaoVw
+Why: The 'Dean of Valuation' posts his entire NYU Stern MBA semester online.
+Highest-signal test — if the first 5 sessions energize you, finance is your field.
+Nothing freely available comes close in rigor or completeness.
+🎯 Careers if it clicks: Investment banking, PE/VC, equity research, asset
+management, corporate development, M&amp;A.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="70" t="inlineStr">
@@ -1506,6 +1608,18 @@
       <c r="L12" s="65" t="inlineStr">
         <is>
           <t>HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
+      <c r="M12" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Microeconomics
+FREE · mru.org
+mru.org/courses/principles-of-microeconomics
+Why: Built by Tyler Cowen (GMU professor) for self-learners — short, vivid,
+real-world examples. Tests whether thinking in incentives and trade-offs excites you.
+Add the Freakonomics Radio podcast (freakonomics.com) for applied macro flavor.
+🎯 Careers if it clicks: Economic consulting, policy/think tanks, central banking,
+pricing strategy, data economics.</t>
         </is>
       </c>
     </row>
@@ -1576,6 +1690,18 @@
 HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M13" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Microeconomics
+FREE · mru.org
+mru.org/courses/principles-of-microeconomics
+Why: Built by Tyler Cowen (GMU professor) for self-learners — short, vivid,
+real-world examples. Tests whether thinking in incentives and trade-offs excites you.
+Add the Freakonomics Radio podcast (freakonomics.com) for applied macro flavor.
+🎯 Careers if it clicks: Economic consulting, policy/think tanks, central banking,
+pricing strategy, data economics.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1644,6 +1770,18 @@
 HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M14" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Microeconomics
+FREE · mru.org
+mru.org/courses/principles-of-microeconomics
+Why: Built by Tyler Cowen (GMU professor) for self-learners — short, vivid,
+real-world examples. Tests whether thinking in incentives and trade-offs excites you.
+Add the Freakonomics Radio podcast (freakonomics.com) for applied macro flavor.
+🎯 Careers if it clicks: Economic consulting, policy/think tanks, central banking,
+pricing strategy, data economics.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1709,6 +1847,18 @@
 Stanford LEAD Program ~$19,200 (gsb.stanford.edu/exec-ed/programs/stanford-lead)
 ★ OTHER PAID:
 HBS Online Economics for Managers (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
+      <c r="M15" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Microeconomics
+FREE · mru.org
+mru.org/courses/principles-of-microeconomics
+Why: Built by Tyler Cowen (GMU professor) for self-learners — short, vivid,
+real-world examples. Tests whether thinking in incentives and trade-offs excites you.
+Add the Freakonomics Radio podcast (freakonomics.com) for applied macro flavor.
+🎯 Careers if it clicks: Economic consulting, policy/think tanks, central banking,
+pricing strategy, data economics.</t>
         </is>
       </c>
     </row>
@@ -1781,6 +1931,18 @@
 — (no direct HBS Online equivalent)</t>
         </is>
       </c>
+      <c r="M16" s="65" t="inlineStr">
+        <is>
+          <t>Marginal Revolution University – Principles of Microeconomics
+FREE · mru.org
+mru.org/courses/principles-of-microeconomics
+Why: Built by Tyler Cowen (GMU professor) for self-learners — short, vivid,
+real-world examples. Tests whether thinking in incentives and trade-offs excites you.
+Add the Freakonomics Radio podcast (freakonomics.com) for applied macro flavor.
+🎯 Careers if it clicks: Economic consulting, policy/think tanks, central banking,
+pricing strategy, data economics.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="72" t="inlineStr">
@@ -1840,6 +2002,19 @@
         <is>
           <t>HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)
 Wharton Marketing on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="M17" s="65" t="inlineStr">
+        <is>
+          <t>HubSpot Academy – Inbound Marketing Certification
+FREE · academy.hubspot.com
+academy.hubspot.com
+Why: Hands-on, immediately career-relevant. You'll know within hours if building
+campaigns and understanding customer behavior excites you.
+Upgrade path: HBS Online Digital Marketing Strategy (~$1,750) with Prof. Sunil
+Gupta for the strategic/brand layer.
+🎯 Careers if it clicks: Brand management, growth marketing, product marketing,
+digital strategy, CMO track.</t>
         </is>
       </c>
     </row>
@@ -1912,6 +2087,19 @@
 HBS Online Digital Marketing Strategy ~$1,750 (online.hbs.edu/courses/digital-marketing-strategy)</t>
         </is>
       </c>
+      <c r="M18" s="65" t="inlineStr">
+        <is>
+          <t>HubSpot Academy – Inbound Marketing Certification
+FREE · academy.hubspot.com
+academy.hubspot.com
+Why: Hands-on, immediately career-relevant. You'll know within hours if building
+campaigns and understanding customer behavior excites you.
+Upgrade path: HBS Online Digital Marketing Strategy (~$1,750) with Prof. Sunil
+Gupta for the strategic/brand layer.
+🎯 Careers if it clicks: Brand management, growth marketing, product marketing,
+digital strategy, CMO track.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -1976,6 +2164,19 @@
 Wharton Marketing on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
+      <c r="M19" s="65" t="inlineStr">
+        <is>
+          <t>HubSpot Academy – Inbound Marketing Certification
+FREE · academy.hubspot.com
+academy.hubspot.com
+Why: Hands-on, immediately career-relevant. You'll know within hours if building
+campaigns and understanding customer behavior excites you.
+Upgrade path: HBS Online Digital Marketing Strategy (~$1,750) with Prof. Sunil
+Gupta for the strategic/brand layer.
+🎯 Careers if it clicks: Brand management, growth marketing, product marketing,
+digital strategy, CMO track.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="74" t="inlineStr">
@@ -2034,6 +2235,18 @@
         <is>
           <t>HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)
 Wharton Operations on Coursera ~$49 cert (coursera.org/specializations/wharton-business-foundations)</t>
+        </is>
+      </c>
+      <c r="M20" s="65" t="inlineStr">
+        <is>
+          <t>MIT OCW 15.761 – Introduction to Operations Management
+FREE · MIT OpenCourseWare
+ocw.mit.edu/courses/15-761-introduction-to-operations-management-spring-2013/
+Why: Supply-chain simulations let you do the work, not just read about it.
+Reveals quickly if optimizing systems and processes is your thing.
+Alternatively: MIT OCW 15.760b (2004 version) for more lecture notes.
+🎯 Careers if it clicks: Supply chain, operations management, consulting,
+manufacturing, logistics, procurement.</t>
         </is>
       </c>
     </row>
@@ -2105,6 +2318,18 @@
 Wharton Operations on Coursera ~$49 cert</t>
         </is>
       </c>
+      <c r="M21" s="65" t="inlineStr">
+        <is>
+          <t>MIT OCW 15.761 – Introduction to Operations Management
+FREE · MIT OpenCourseWare
+ocw.mit.edu/courses/15-761-introduction-to-operations-management-spring-2013/
+Why: Supply-chain simulations let you do the work, not just read about it.
+Reveals quickly if optimizing systems and processes is your thing.
+Alternatively: MIT OCW 15.760b (2004 version) for more lecture notes.
+🎯 Careers if it clicks: Supply chain, operations management, consulting,
+manufacturing, logistics, procurement.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
@@ -2167,6 +2392,18 @@
 HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
         </is>
       </c>
+      <c r="M22" s="65" t="inlineStr">
+        <is>
+          <t>MIT OCW 15.761 – Introduction to Operations Management
+FREE · MIT OpenCourseWare
+ocw.mit.edu/courses/15-761-introduction-to-operations-management-spring-2013/
+Why: Supply-chain simulations let you do the work, not just read about it.
+Reveals quickly if optimizing systems and processes is your thing.
+Alternatively: MIT OCW 15.760b (2004 version) for more lecture notes.
+🎯 Careers if it clicks: Supply chain, operations management, consulting,
+manufacturing, logistics, procurement.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="76" t="inlineStr">
@@ -2230,6 +2467,18 @@
         <is>
           <t>HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)
 HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
+      <c r="M23" s="65" t="inlineStr">
+        <is>
+          <t>Alex The Analyst – Data Analyst Bootcamp ⭐
+FREE · YouTube
+youtube.com/@AlexTheAnalyst
+Why: Career-shaped from day one: SQL → Python → Power BI → portfolio.
+Quickly reveals if working with data day-to-day clicks for you.
+Pair with StatQuest (youtube.com/c/joshstarmer) if the ML/AI layer pulls you deeper.
+🎯 Careers if it clicks: Data analyst, business intelligence, data science,
+analytics consulting, AI product roles.</t>
         </is>
       </c>
     </row>
@@ -2301,6 +2550,18 @@
 HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
         </is>
       </c>
+      <c r="M24" s="65" t="inlineStr">
+        <is>
+          <t>Alex The Analyst – Data Analyst Bootcamp ⭐
+FREE · YouTube
+youtube.com/@AlexTheAnalyst
+Why: Career-shaped from day one: SQL → Python → Power BI → portfolio.
+Quickly reveals if working with data day-to-day clicks for you.
+Pair with StatQuest (youtube.com/c/joshstarmer) if the ML/AI layer pulls you deeper.
+🎯 Careers if it clicks: Data analyst, business intelligence, data science,
+analytics consulting, AI product roles.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -2369,6 +2630,18 @@
 HBS Online Business Analytics (part of CORe ~$2,650; online.hbs.edu/courses/core)</t>
         </is>
       </c>
+      <c r="M25" s="65" t="inlineStr">
+        <is>
+          <t>Alex The Analyst – Data Analyst Bootcamp ⭐
+FREE · YouTube
+youtube.com/@AlexTheAnalyst
+Why: Career-shaped from day one: SQL → Python → Power BI → portfolio.
+Quickly reveals if working with data day-to-day clicks for you.
+Pair with StatQuest (youtube.com/c/joshstarmer) if the ML/AI layer pulls you deeper.
+🎯 Careers if it clicks: Data analyst, business intelligence, data science,
+analytics consulting, AI product roles.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -2429,6 +2702,18 @@
 Stanford GSB Demystify Decision Making (gsb.stanford.edu/exec-ed/programs/demystify-decision-making)
 ★ OTHER PAID:
 HBS Online Data Science &amp; AI for Decision Making (online.hbs.edu/courses/data-science-ai-decision-making)</t>
+        </is>
+      </c>
+      <c r="M26" s="65" t="inlineStr">
+        <is>
+          <t>Alex The Analyst – Data Analyst Bootcamp ⭐
+FREE · YouTube
+youtube.com/@AlexTheAnalyst
+Why: Career-shaped from day one: SQL → Python → Power BI → portfolio.
+Quickly reveals if working with data day-to-day clicks for you.
+Pair with StatQuest (youtube.com/c/joshstarmer) if the ML/AI layer pulls you deeper.
+🎯 Careers if it clicks: Data analyst, business intelligence, data science,
+analytics consulting, AI product roles.</t>
         </is>
       </c>
     </row>
@@ -2494,6 +2779,18 @@
 — (no direct HBS Online equivalent)</t>
         </is>
       </c>
+      <c r="M27" s="65" t="inlineStr">
+        <is>
+          <t>Alex The Analyst – Data Analyst Bootcamp ⭐
+FREE · YouTube
+youtube.com/@AlexTheAnalyst
+Why: Career-shaped from day one: SQL → Python → Power BI → portfolio.
+Quickly reveals if working with data day-to-day clicks for you.
+Pair with StatQuest (youtube.com/c/joshstarmer) if the ML/AI layer pulls you deeper.
+🎯 Careers if it clicks: Data analyst, business intelligence, data science,
+analytics consulting, AI product roles.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="78" t="inlineStr">
@@ -2554,6 +2851,19 @@
         <is>
           <t>HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)
 HBS Online Core Business Essentials ~$2,650 – includes Strategy module (online.hbs.edu/courses/core)</t>
+        </is>
+      </c>
+      <c r="M28" s="65" t="inlineStr">
+        <is>
+          <t>Modern MBA – Company Case Studies ⭐
+FREE · YouTube
+youtube.com/c/ModernMBA
+Why: Emmy-quality 40-min deep-dives on real companies (Apple, Netflix, LVMH…).
+The closest free equivalent to the HBS case method. If you binge these,
+strategy is your field. Pair with the Acquired Podcast (acquired.fm) for
+narrative-style company histories.
+🎯 Careers if it clicks: Management consulting (MBB), corporate strategy,
+BizOps, M&amp;A, general management.</t>
         </is>
       </c>
     </row>
@@ -2627,6 +2937,19 @@
 Wharton Business Foundations on Coursera – free audit (coursera.org/specializations/wharton-business-foundations)</t>
         </is>
       </c>
+      <c r="M29" s="65" t="inlineStr">
+        <is>
+          <t>Modern MBA – Company Case Studies ⭐
+FREE · YouTube
+youtube.com/c/ModernMBA
+Why: Emmy-quality 40-min deep-dives on real companies (Apple, Netflix, LVMH…).
+The closest free equivalent to the HBS case method. If you binge these,
+strategy is your field. Pair with the Acquired Podcast (acquired.fm) for
+narrative-style company histories.
+🎯 Careers if it clicks: Management consulting (MBB), corporate strategy,
+BizOps, M&amp;A, general management.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
@@ -2694,6 +3017,19 @@
 HBS Online Disruptive Strategy ~$1,949 (online.hbs.edu/courses/disruptive-strategy)</t>
         </is>
       </c>
+      <c r="M30" s="65" t="inlineStr">
+        <is>
+          <t>Modern MBA – Company Case Studies ⭐
+FREE · YouTube
+youtube.com/c/ModernMBA
+Why: Emmy-quality 40-min deep-dives on real companies (Apple, Netflix, LVMH…).
+The closest free equivalent to the HBS case method. If you binge these,
+strategy is your field. Pair with the Acquired Podcast (acquired.fm) for
+narrative-style company histories.
+🎯 Careers if it clicks: Management consulting (MBB), corporate strategy,
+BizOps, M&amp;A, general management.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="80" t="inlineStr">
@@ -2755,6 +3091,18 @@
         <is>
           <t>HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)
 HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
+        </is>
+      </c>
+      <c r="M31" s="65" t="inlineStr">
+        <is>
+          <t>Coursera – Organizational Analysis (Stanford University)
+FREE audit · coursera.org
+coursera.org/learn/organizational-analysis
+Why: A genuine Stanford academic course (4.6★, 78,000+ learners).
+Tests whether the theory of how organizations and people behave fascinates
+you — beyond 'leadership is inspiring' to the real science behind it.
+🎯 Careers if it clicks: HR / People leadership, org design, talent,
+executive coaching, organizational consulting.</t>
         </is>
       </c>
     </row>
@@ -2826,6 +3174,18 @@
 HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
         </is>
       </c>
+      <c r="M32" s="65" t="inlineStr">
+        <is>
+          <t>Coursera – Organizational Analysis (Stanford University)
+FREE audit · coursera.org
+coursera.org/learn/organizational-analysis
+Why: A genuine Stanford academic course (4.6★, 78,000+ learners).
+Tests whether the theory of how organizations and people behave fascinates
+you — beyond 'leadership is inspiring' to the real science behind it.
+🎯 Careers if it clicks: HR / People leadership, org design, talent,
+executive coaching, organizational consulting.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -2895,6 +3255,18 @@
 HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
         </is>
       </c>
+      <c r="M33" s="65" t="inlineStr">
+        <is>
+          <t>Coursera – Organizational Analysis (Stanford University)
+FREE audit · coursera.org
+coursera.org/learn/organizational-analysis
+Why: A genuine Stanford academic course (4.6★, 78,000+ learners).
+Tests whether the theory of how organizations and people behave fascinates
+you — beyond 'leadership is inspiring' to the real science behind it.
+🎯 Careers if it clicks: HR / People leadership, org design, talent,
+executive coaching, organizational consulting.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
@@ -2958,6 +3330,18 @@
 HBS Online Management Essentials ~$1,750 (online.hbs.edu/courses/management-essentials)</t>
         </is>
       </c>
+      <c r="M34" s="65" t="inlineStr">
+        <is>
+          <t>Coursera – Organizational Analysis (Stanford University)
+FREE audit · coursera.org
+coursera.org/learn/organizational-analysis
+Why: A genuine Stanford academic course (4.6★, 78,000+ learners).
+Tests whether the theory of how organizations and people behave fascinates
+you — beyond 'leadership is inspiring' to the real science behind it.
+🎯 Careers if it clicks: HR / People leadership, org design, talent,
+executive coaching, organizational consulting.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="82" t="inlineStr">
@@ -3019,6 +3403,19 @@
           <t>HBS Online Negotiation Mastery ~$1,850 (online.hbs.edu/courses/negotiation)</t>
         </is>
       </c>
+      <c r="M35" s="65" t="inlineStr">
+        <is>
+          <t>Michael Sandel – Justice (Harvard University)
+FREE · YouTube / justiceharvard.org
+justiceharvard.org
+Why: Harvard's legendary ethics course — the best free test of whether
+moral reasoning genuinely grips you. For the business ethics angle, browse
+Stanford Social Innovation Review (ssir.org) — free articles on ESG,
+stakeholder capitalism, and corporate accountability.
+🎯 Careers if it clicks: ESG / sustainability, corporate responsibility,
+compliance, social enterprise, impact investing.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -3077,6 +3474,19 @@
       <c r="L36" s="65" t="inlineStr">
         <is>
           <t>— (no direct HBS Online equivalent)</t>
+        </is>
+      </c>
+      <c r="M36" s="65" t="inlineStr">
+        <is>
+          <t>Michael Sandel – Justice (Harvard University)
+FREE · YouTube / justiceharvard.org
+justiceharvard.org
+Why: Harvard's legendary ethics course — the best free test of whether
+moral reasoning genuinely grips you. For the business ethics angle, browse
+Stanford Social Innovation Review (ssir.org) — free articles on ESG,
+stakeholder capitalism, and corporate accountability.
+🎯 Careers if it clicks: ESG / sustainability, corporate responsibility,
+compliance, social enterprise, impact investing.</t>
         </is>
       </c>
     </row>
@@ -3143,6 +3553,19 @@
 — (no direct HBS Online equivalent)</t>
         </is>
       </c>
+      <c r="M37" s="65" t="inlineStr">
+        <is>
+          <t>Michael Sandel – Justice (Harvard University)
+FREE · YouTube / justiceharvard.org
+justiceharvard.org
+Why: Harvard's legendary ethics course — the best free test of whether
+moral reasoning genuinely grips you. For the business ethics angle, browse
+Stanford Social Innovation Review (ssir.org) — free articles on ESG,
+stakeholder capitalism, and corporate accountability.
+🎯 Careers if it clicks: ESG / sustainability, corporate responsibility,
+compliance, social enterprise, impact investing.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="84" t="inlineStr">
@@ -3205,6 +3628,18 @@
       <c r="L38" s="65" t="inlineStr">
         <is>
           <t>HBS Online Entrepreneurship Essentials ~$1,850 (online.hbs.edu/courses/entrepreneurship-essentials)</t>
+        </is>
+      </c>
+      <c r="M38" s="65" t="inlineStr">
+        <is>
+          <t>Y Combinator – Startup School ⭐
+FREE · Structured Curriculum
+startupschool.org/curriculum
+Why: Taught by YC partners who funded Airbnb, Stripe, Dropbox, Coinbase.
+Dense, practical, zero fluff. You'll know within the first 3 sessions
+whether the founder path actually calls you.
+🎯 Careers if it clicks: Founder, early startup operator, VC/angel investing,
+product management, intrapreneurship.</t>
         </is>
       </c>
     </row>
@@ -3278,6 +3713,20 @@
 — (no direct HBS Online equivalent)</t>
         </is>
       </c>
+      <c r="M39" s="65" t="inlineStr">
+        <is>
+          <t>Think Fast, Talk Smart – Podcast (Stanford GSB)
+FREE · 200+ episodes
+gsb.stanford.edu/business-podcasts/think-fast-talk-smart-podcast
+fastersmarter.io
+Why: Matt Abrahams (Stanford GSB) covers communication anxiety, impromptu
+speaking, persuasion, negotiation presence. Immediately applicable.
+Note: Communication is a career multiplier, not a standalone field — it
+compounds every other career path you choose.
+🎯 Where it helps most: Leadership, consulting, sales, investor relations,
+any exec-track role.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="88" t="inlineStr">
@@ -3338,6 +3787,20 @@
       <c r="L40" s="65" t="inlineStr">
         <is>
           <t>— (experiential program; no direct online equivalent)</t>
+        </is>
+      </c>
+      <c r="M40" s="65" t="inlineStr">
+        <is>
+          <t>Stanford eCorner – Entrepreneurial Thought Leaders Series
+FREE · 2,000+ videos
+ecorner.stanford.edu
+youtube.com/@ecorner
+Why: The best free taste of global business, cross-border entrepreneurship,
+and international strategy. Guests include founders, VCs, and operators from
+90+ countries. Experiential learning has no true online substitute, but
+eCorner's global founder stories give you the flavor of international careers.
+🎯 Careers if it clicks: International business development, global strategy,
+cross-border M&amp;A, emerging markets, development finance.</t>
         </is>
       </c>
     </row>
@@ -3396,6 +3859,20 @@
       <c r="L41" s="65" t="inlineStr">
         <is>
           <t>— (experiential / global immersion; no direct online equivalent)</t>
+        </is>
+      </c>
+      <c r="M41" s="65" t="inlineStr">
+        <is>
+          <t>Stanford eCorner – Entrepreneurial Thought Leaders Series
+FREE · 2,000+ videos
+ecorner.stanford.edu
+youtube.com/@ecorner
+Why: The best free taste of global business, cross-border entrepreneurship,
+and international strategy. Guests include founders, VCs, and operators from
+90+ countries. Experiential learning has no true online substitute, but
+eCorner's global founder stories give you the flavor of international careers.
+🎯 Careers if it clicks: International business development, global strategy,
+cross-border M&amp;A, emerging markets, development finance.</t>
         </is>
       </c>
     </row>
@@ -3466,6 +3943,20 @@
 — (immersive off-campus; no direct online equivalent)</t>
         </is>
       </c>
+      <c r="M42" s="65" t="inlineStr">
+        <is>
+          <t>Stanford eCorner – Entrepreneurial Thought Leaders Series
+FREE · 2,000+ videos
+ecorner.stanford.edu
+youtube.com/@ecorner
+Why: The best free taste of global business, cross-border entrepreneurship,
+and international strategy. Guests include founders, VCs, and operators from
+90+ countries. Experiential learning has no true online substitute, but
+eCorner's global founder stories give you the flavor of international careers.
+🎯 Careers if it clicks: International business development, global strategy,
+cross-border M&amp;A, emerging markets, development finance.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -3532,6 +4023,20 @@
 HBS Online Leadership Principles ~$1,850 (online.hbs.edu/courses/leadership-principles)</t>
         </is>
       </c>
+      <c r="M43" s="65" t="inlineStr">
+        <is>
+          <t>Stanford eCorner – Entrepreneurial Thought Leaders Series
+FREE · 2,000+ videos
+ecorner.stanford.edu
+youtube.com/@ecorner
+Why: The best free taste of global business, cross-border entrepreneurship,
+and international strategy. Guests include founders, VCs, and operators from
+90+ countries. Experiential learning has no true online substitute, but
+eCorner's global founder stories give you the flavor of international careers.
+🎯 Careers if it clicks: International business development, global strategy,
+cross-border M&amp;A, emerging markets, development finance.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n"/>
@@ -3596,6 +4101,20 @@
 Stanford LEAD Program ~$19,200 – global cohort &amp; virtual immersion (gsb.stanford.edu/exec-ed/programs/stanford-lead)
 ★ OTHER PAID:
 — (global immersion requirement; no direct online equivalent)</t>
+        </is>
+      </c>
+      <c r="M44" s="65" t="inlineStr">
+        <is>
+          <t>Stanford eCorner – Entrepreneurial Thought Leaders Series
+FREE · 2,000+ videos
+ecorner.stanford.edu
+youtube.com/@ecorner
+Why: The best free taste of global business, cross-border entrepreneurship,
+and international strategy. Guests include founders, VCs, and operators from
+90+ countries. Experiential learning has no true online substitute, but
+eCorner's global founder stories give you the flavor of international careers.
+🎯 Careers if it clicks: International business development, global strategy,
+cross-border M&amp;A, emerging markets, development finance.</t>
         </is>
       </c>
     </row>

</xml_diff>